<commit_message>
pushing after a while
</commit_message>
<xml_diff>
--- a/experiments/notebooks/results/summarized/summarized_fs_dynamic_bootstrapping_ss_None_sp_None.xlsx
+++ b/experiments/notebooks/results/summarized/summarized_fs_dynamic_bootstrapping_ss_None_sp_None.xlsx
@@ -677,64 +677,64 @@
         <v>1</v>
       </c>
       <c r="C7" s="4">
-        <v>0.2348497854077253</v>
+        <v>0.2338197424892704</v>
       </c>
       <c r="D7" s="4">
-        <v>0.5351851851851851</v>
+        <v>0.4318287037037036</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F7" s="5">
-        <v>0.2270462633451957</v>
+        <v>1</v>
       </c>
       <c r="G7" s="5">
-        <v>0.9982832618025752</v>
+        <v>0.2345064377682403</v>
       </c>
       <c r="H7" s="5">
-        <v>0.2543402777777778</v>
+        <v>0.4340856481481482</v>
       </c>
       <c r="I7" s="5">
-        <v>-0.7729537366548043</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5">
-        <v>0.7634334763948499</v>
+        <v>0.0006866952789699732</v>
       </c>
       <c r="K7" s="5">
-        <v>-0.2808449074074073</v>
+        <v>0.002256944444444575</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N7" s="4">
-        <v>0.9992882562277579</v>
+        <v>1</v>
       </c>
       <c r="O7" s="4">
-        <v>0.4097854077253219</v>
+        <v>0.4039484978540773</v>
       </c>
       <c r="P7" s="4">
-        <v>0.441724537037037</v>
+        <v>0.4416666666666667</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>9</v>
       </c>
       <c r="R7" s="5">
-        <v>0.4384341637010676</v>
+        <v>1</v>
       </c>
       <c r="S7" s="5">
-        <v>0.9656652360515021</v>
+        <v>0.3986266094420601</v>
       </c>
       <c r="T7" s="5">
-        <v>0.3593171296296296</v>
+        <v>0.439699074074074</v>
       </c>
       <c r="U7" s="5">
-        <v>-0.5608540925266903</v>
+        <v>0</v>
       </c>
       <c r="V7" s="5">
-        <v>0.5558798283261802</v>
+        <v>-0.005321888412017195</v>
       </c>
       <c r="W7" s="5">
-        <v>-0.08240740740740737</v>
+        <v>-0.00196759259259266</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -746,22 +746,22 @@
         <v>10</v>
       </c>
       <c r="F8" s="5">
-        <v>0.6903914590747331</v>
+        <v>1</v>
       </c>
       <c r="G8" s="5">
-        <v>0.1526180257510729</v>
+        <v>0.232618025751073</v>
       </c>
       <c r="H8" s="5">
-        <v>1</v>
+        <v>0.4309606481481482</v>
       </c>
       <c r="I8" s="5">
-        <v>-0.3096085409252669</v>
+        <v>0</v>
       </c>
       <c r="J8" s="5">
-        <v>-0.08223175965665236</v>
+        <v>-0.001201716738197411</v>
       </c>
       <c r="K8" s="5">
-        <v>0.4648148148148149</v>
+        <v>-0.0008680555555554692</v>
       </c>
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
@@ -771,22 +771,22 @@
         <v>10</v>
       </c>
       <c r="R8" s="5">
-        <v>0.5039145907473309</v>
+        <v>1</v>
       </c>
       <c r="S8" s="5">
-        <v>0.3907296137339056</v>
+        <v>0.4051502145922747</v>
       </c>
       <c r="T8" s="5">
-        <v>0.9997685185185186</v>
+        <v>0.4411458333333334</v>
       </c>
       <c r="U8" s="5">
-        <v>-0.4953736654804269</v>
+        <v>0</v>
       </c>
       <c r="V8" s="5">
-        <v>-0.01905579399141633</v>
+        <v>0.001201716738197411</v>
       </c>
       <c r="W8" s="5">
-        <v>0.5580439814814815</v>
+        <v>-0.0005208333333333037</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -794,67 +794,67 @@
         <v>9</v>
       </c>
       <c r="B9" s="4">
-        <v>0.2733096085409253</v>
+        <v>0.2775800711743773</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
       </c>
       <c r="D9" s="4">
-        <v>0.2195023148148148</v>
+        <v>0.2764467592592593</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F9" s="5">
-        <v>1</v>
+        <v>0.2775800711743773</v>
       </c>
       <c r="G9" s="5">
-        <v>0.4044635193133048</v>
+        <v>0.999656652360515</v>
       </c>
       <c r="H9" s="5">
-        <v>0.4499421296296296</v>
+        <v>0.2730324074074074</v>
       </c>
       <c r="I9" s="5">
-        <v>0.7266903914590748</v>
+        <v>0</v>
       </c>
       <c r="J9" s="5">
-        <v>-0.5955364806866952</v>
+        <v>-0.0003433476394849588</v>
       </c>
       <c r="K9" s="5">
-        <v>0.2304398148148148</v>
+        <v>-0.003414351851851849</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N9" s="4">
-        <v>0.4384341637010676</v>
+        <v>0.4192170818505338</v>
       </c>
       <c r="O9" s="4">
-        <v>0.9970815450643776</v>
+        <v>0.9921030042918455</v>
       </c>
       <c r="P9" s="4">
-        <v>0.404050925925926</v>
+        <v>0.4226851851851851</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R9" s="5">
-        <v>1</v>
+        <v>0.4163701067615658</v>
       </c>
       <c r="S9" s="5">
-        <v>0.4769098712446351</v>
+        <v>0.9917596566523604</v>
       </c>
       <c r="T9" s="5">
-        <v>0.4426504629629631</v>
+        <v>0.4265625</v>
       </c>
       <c r="U9" s="5">
-        <v>0.5615658362989324</v>
+        <v>-0.002846975088967973</v>
       </c>
       <c r="V9" s="5">
-        <v>-0.5201716738197425</v>
+        <v>-0.0003433476394850699</v>
       </c>
       <c r="W9" s="5">
-        <v>0.03859953703703711</v>
+        <v>0.003877314814814903</v>
       </c>
     </row>
     <row r="10" spans="1:23">
@@ -866,22 +866,22 @@
         <v>10</v>
       </c>
       <c r="F10" s="5">
-        <v>0.505338078291815</v>
+        <v>0.2747330960854092</v>
       </c>
       <c r="G10" s="5">
-        <v>0.4199141630901287</v>
+        <v>1</v>
       </c>
       <c r="H10" s="5">
-        <v>1</v>
+        <v>0.2733796296296296</v>
       </c>
       <c r="I10" s="5">
-        <v>0.2320284697508897</v>
+        <v>-0.002846975088968029</v>
       </c>
       <c r="J10" s="5">
-        <v>-0.5800858369098713</v>
+        <v>0</v>
       </c>
       <c r="K10" s="5">
-        <v>0.7804976851851853</v>
+        <v>-0.003067129629629628</v>
       </c>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
@@ -891,22 +891,22 @@
         <v>10</v>
       </c>
       <c r="R10" s="5">
-        <v>0.4996441281138789</v>
+        <v>0.4234875444839857</v>
       </c>
       <c r="S10" s="5">
-        <v>0.3745922746781116</v>
+        <v>0.9917596566523604</v>
       </c>
       <c r="T10" s="5">
-        <v>0.9999421296296296</v>
+        <v>0.4234953703703703</v>
       </c>
       <c r="U10" s="5">
-        <v>0.06120996441281129</v>
+        <v>0.004270462633451932</v>
       </c>
       <c r="V10" s="5">
-        <v>-0.6224892703862661</v>
+        <v>-0.0003433476394850699</v>
       </c>
       <c r="W10" s="5">
-        <v>0.5958912037037036</v>
+        <v>0.0008101851851852193</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -914,10 +914,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="4">
-        <v>0.510320284697509</v>
+        <v>0.5046263345195729</v>
       </c>
       <c r="C11" s="4">
-        <v>0.3096995708154506</v>
+        <v>0.2626609442060086</v>
       </c>
       <c r="D11" s="4">
         <v>1</v>
@@ -926,55 +926,55 @@
         <v>8</v>
       </c>
       <c r="F11" s="5">
+        <v>0.5046263345195729</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0.2684978540772532</v>
+      </c>
+      <c r="H11" s="5">
         <v>1</v>
       </c>
-      <c r="G11" s="5">
-        <v>0.2149356223175966</v>
-      </c>
-      <c r="H11" s="5">
-        <v>0.6940972222222224</v>
-      </c>
       <c r="I11" s="5">
-        <v>0.489679715302491</v>
+        <v>0</v>
       </c>
       <c r="J11" s="5">
-        <v>-0.09476394849785405</v>
+        <v>0.005836909871244633</v>
       </c>
       <c r="K11" s="5">
-        <v>-0.3059027777777776</v>
+        <v>0</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N11" s="4">
-        <v>0.502491103202847</v>
+        <v>0.4967971530249111</v>
       </c>
       <c r="O11" s="4">
-        <v>0.4607725321888412</v>
+        <v>0.4115021459227467</v>
       </c>
       <c r="P11" s="4">
-        <v>0.999826388888889</v>
+        <v>0.9999421296296296</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R11" s="5">
-        <v>0.9907473309608541</v>
+        <v>0.4967971530249111</v>
       </c>
       <c r="S11" s="5">
-        <v>0.471587982832618</v>
+        <v>0.4142489270386266</v>
       </c>
       <c r="T11" s="5">
-        <v>0.4821180555555555</v>
+        <v>1</v>
       </c>
       <c r="U11" s="5">
-        <v>0.4882562277580071</v>
+        <v>0</v>
       </c>
       <c r="V11" s="5">
-        <v>0.01081545064377681</v>
+        <v>0.002746781115879893</v>
       </c>
       <c r="W11" s="5">
-        <v>-0.5177083333333334</v>
+        <v>5.787037037041642E-05</v>
       </c>
     </row>
     <row r="12" spans="1:23">
@@ -986,22 +986,22 @@
         <v>9</v>
       </c>
       <c r="F12" s="5">
-        <v>0.3024911032028469</v>
+        <v>0.5046263345195729</v>
       </c>
       <c r="G12" s="5">
-        <v>0.9934763948497853</v>
+        <v>0.264549356223176</v>
       </c>
       <c r="H12" s="5">
-        <v>0.3335648148148148</v>
+        <v>1</v>
       </c>
       <c r="I12" s="5">
-        <v>-0.2078291814946621</v>
+        <v>0</v>
       </c>
       <c r="J12" s="5">
-        <v>0.6837768240343347</v>
+        <v>0.001888412017167385</v>
       </c>
       <c r="K12" s="5">
-        <v>-0.6664351851851852</v>
+        <v>0</v>
       </c>
       <c r="M12" s="4"/>
       <c r="N12" s="4"/>
@@ -1011,22 +1011,22 @@
         <v>9</v>
       </c>
       <c r="R12" s="5">
-        <v>0.3366548042704626</v>
+        <v>0.4967971530249111</v>
       </c>
       <c r="S12" s="5">
-        <v>0.9234334763948496</v>
+        <v>0.4120171673819742</v>
       </c>
       <c r="T12" s="5">
-        <v>0.6515046296296296</v>
+        <v>1</v>
       </c>
       <c r="U12" s="5">
-        <v>-0.1658362989323843</v>
+        <v>0</v>
       </c>
       <c r="V12" s="5">
-        <v>0.4626609442060084</v>
+        <v>0.0005150214592275493</v>
       </c>
       <c r="W12" s="5">
-        <v>-0.3483217592592593</v>
+        <v>5.787037037041642E-05</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -1195,64 +1195,64 @@
         <v>1</v>
       </c>
       <c r="C25" s="4">
-        <v>0.1859227467811159</v>
+        <v>0.2099570815450644</v>
       </c>
       <c r="D25" s="4">
-        <v>0.3929976851851852</v>
+        <v>0.3939814814814815</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F25" s="5">
-        <v>0.7587188612099645</v>
+        <v>1</v>
       </c>
       <c r="G25" s="5">
-        <v>1</v>
+        <v>0.2096137339055794</v>
       </c>
       <c r="H25" s="5">
-        <v>0.3333912037037037</v>
+        <v>0.3950810185185186</v>
       </c>
       <c r="I25" s="5">
-        <v>-0.2412811387900355</v>
+        <v>0</v>
       </c>
       <c r="J25" s="5">
-        <v>0.8140772532188841</v>
+        <v>-0.0003433476394849866</v>
       </c>
       <c r="K25" s="5">
-        <v>-0.05960648148148145</v>
+        <v>0.001099537037037079</v>
       </c>
       <c r="M25" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N25" s="4">
-        <v>0.9957295373665479</v>
+        <v>0.99644128113879</v>
       </c>
       <c r="O25" s="4">
-        <v>0.6066952789699571</v>
+        <v>0.5795708154506437</v>
       </c>
       <c r="P25" s="4">
-        <v>0.4179976851851851</v>
+        <v>0.4256365740740741</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="R25" s="5">
-        <v>0.6199288256227758</v>
+        <v>0.9943060498220641</v>
       </c>
       <c r="S25" s="5">
-        <v>0.9507296137339056</v>
+        <v>0.5809442060085838</v>
       </c>
       <c r="T25" s="5">
-        <v>0.4867476851851852</v>
+        <v>0.4244791666666667</v>
       </c>
       <c r="U25" s="5">
-        <v>-0.3758007117437721</v>
+        <v>-0.002135231316725994</v>
       </c>
       <c r="V25" s="5">
-        <v>0.3440343347639485</v>
+        <v>0.001373390557940057</v>
       </c>
       <c r="W25" s="5">
-        <v>0.06875000000000009</v>
+        <v>-0.001157407407407385</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -1264,22 +1264,22 @@
         <v>10</v>
       </c>
       <c r="F26" s="5">
-        <v>0.5836298932384342</v>
+        <v>1</v>
       </c>
       <c r="G26" s="5">
-        <v>0.3076394849785408</v>
+        <v>0.1989699570815451</v>
       </c>
       <c r="H26" s="5">
-        <v>1</v>
+        <v>0.3929398148148148</v>
       </c>
       <c r="I26" s="5">
-        <v>-0.4163701067615658</v>
+        <v>0</v>
       </c>
       <c r="J26" s="5">
-        <v>0.1217167381974249</v>
+        <v>-0.01098712446351932</v>
       </c>
       <c r="K26" s="5">
-        <v>0.6070023148148148</v>
+        <v>-0.001041666666666718</v>
       </c>
       <c r="M26" s="4"/>
       <c r="N26" s="4"/>
@@ -1289,22 +1289,22 @@
         <v>10</v>
       </c>
       <c r="R26" s="5">
-        <v>0.2911032028469751</v>
+        <v>0.99644128113879</v>
       </c>
       <c r="S26" s="5">
-        <v>0.3086695278969956</v>
+        <v>0.5833476394849785</v>
       </c>
       <c r="T26" s="5">
-        <v>1</v>
+        <v>0.4302662037037036</v>
       </c>
       <c r="U26" s="5">
-        <v>-0.7046263345195729</v>
+        <v>0</v>
       </c>
       <c r="V26" s="5">
-        <v>-0.2980257510729615</v>
+        <v>0.003776824034334769</v>
       </c>
       <c r="W26" s="5">
-        <v>0.5820023148148149</v>
+        <v>0.004629629629629539</v>
       </c>
     </row>
     <row r="27" spans="1:23">
@@ -1312,67 +1312,67 @@
         <v>9</v>
       </c>
       <c r="B27" s="4">
-        <v>0.3857651245551601</v>
+        <v>0.3487544483985766</v>
       </c>
       <c r="C27" s="4">
         <v>0.999656652360515</v>
       </c>
       <c r="D27" s="4">
-        <v>0.4237847222222222</v>
+        <v>0.4013888888888889</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F27" s="5">
-        <v>0.995017793594306</v>
+        <v>0.3480427046263345</v>
       </c>
       <c r="G27" s="5">
-        <v>0.3237768240343348</v>
+        <v>0.999656652360515</v>
       </c>
       <c r="H27" s="5">
-        <v>0.4493055555555555</v>
+        <v>0.3971064814814815</v>
       </c>
       <c r="I27" s="5">
-        <v>0.6092526690391459</v>
+        <v>-0.000711743772242035</v>
       </c>
       <c r="J27" s="5">
-        <v>-0.6758798283261802</v>
+        <v>0</v>
       </c>
       <c r="K27" s="5">
-        <v>0.02552083333333327</v>
+        <v>-0.004282407407407429</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N27" s="4">
-        <v>0.4555160142348755</v>
+        <v>0.5295373665480427</v>
       </c>
       <c r="O27" s="4">
-        <v>0.9649785407725322</v>
+        <v>0.9627467811158799</v>
       </c>
       <c r="P27" s="4">
-        <v>0.3722222222222222</v>
+        <v>0.3358217592592593</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R27" s="5">
-        <v>0.9736654804270464</v>
+        <v>0.5430604982206406</v>
       </c>
       <c r="S27" s="5">
-        <v>0.6848068669527897</v>
+        <v>0.9625751072961373</v>
       </c>
       <c r="T27" s="5">
-        <v>0.5373842592592594</v>
+        <v>0.3316550925925926</v>
       </c>
       <c r="U27" s="5">
-        <v>0.5181494661921708</v>
+        <v>0.01352313167259789</v>
       </c>
       <c r="V27" s="5">
-        <v>-0.2801716738197425</v>
+        <v>-0.0001716738197425904</v>
       </c>
       <c r="W27" s="5">
-        <v>0.1651620370370371</v>
+        <v>-0.004166666666666707</v>
       </c>
     </row>
     <row r="28" spans="1:23">
@@ -1384,22 +1384,22 @@
         <v>10</v>
       </c>
       <c r="F28" s="5">
-        <v>0.3779359430604982</v>
+        <v>0.3473309608540925</v>
       </c>
       <c r="G28" s="5">
-        <v>0.5732188841201717</v>
+        <v>0.999656652360515</v>
       </c>
       <c r="H28" s="5">
-        <v>1</v>
+        <v>0.4049189814814815</v>
       </c>
       <c r="I28" s="5">
-        <v>-0.007829181494661885</v>
+        <v>-0.00142348754448407</v>
       </c>
       <c r="J28" s="5">
-        <v>-0.4264377682403433</v>
+        <v>0</v>
       </c>
       <c r="K28" s="5">
-        <v>0.5762152777777778</v>
+        <v>0.003530092592592571</v>
       </c>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>
@@ -1409,22 +1409,22 @@
         <v>10</v>
       </c>
       <c r="R28" s="5">
-        <v>0.2277580071174377</v>
+        <v>0.5231316725978647</v>
       </c>
       <c r="S28" s="5">
-        <v>0.3167381974248927</v>
+        <v>0.9636051502145924</v>
       </c>
       <c r="T28" s="5">
-        <v>1</v>
+        <v>0.3303819444444445</v>
       </c>
       <c r="U28" s="5">
-        <v>-0.2277580071174377</v>
+        <v>-0.006405693950177982</v>
       </c>
       <c r="V28" s="5">
-        <v>-0.6482403433476395</v>
+        <v>0.0008583690987125081</v>
       </c>
       <c r="W28" s="5">
-        <v>0.6277777777777778</v>
+        <v>-0.005439814814814814</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -1432,10 +1432,10 @@
         <v>10</v>
       </c>
       <c r="B29" s="4">
-        <v>0.4249110320284697</v>
+        <v>0.4476868327402135</v>
       </c>
       <c r="C29" s="4">
-        <v>0.4607725321888412</v>
+        <v>0.5009442060085838</v>
       </c>
       <c r="D29" s="4">
         <v>1</v>
@@ -1444,31 +1444,31 @@
         <v>8</v>
       </c>
       <c r="F29" s="5">
-        <v>0.9992882562277579</v>
+        <v>0.4462633451957295</v>
       </c>
       <c r="G29" s="5">
-        <v>0.2475536480686695</v>
+        <v>0.5012875536480687</v>
       </c>
       <c r="H29" s="5">
-        <v>0.579861111111111</v>
+        <v>1</v>
       </c>
       <c r="I29" s="5">
-        <v>0.5743772241992882</v>
+        <v>-0.001423487544484014</v>
       </c>
       <c r="J29" s="5">
-        <v>-0.2132188841201717</v>
+        <v>0.0003433476394848478</v>
       </c>
       <c r="K29" s="5">
-        <v>-0.420138888888889</v>
+        <v>0</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N29" s="4">
-        <v>0.2199288256227758</v>
+        <v>0.2875444839857652</v>
       </c>
       <c r="O29" s="4">
-        <v>0.336480686695279</v>
+        <v>0.3301287553648068</v>
       </c>
       <c r="P29" s="4">
         <v>1</v>
@@ -1477,22 +1477,22 @@
         <v>8</v>
       </c>
       <c r="R29" s="5">
-        <v>0.9508896797153025</v>
+        <v>0.2825622775800712</v>
       </c>
       <c r="S29" s="5">
-        <v>0.4758798283261802</v>
+        <v>0.3278969957081545</v>
       </c>
       <c r="T29" s="5">
-        <v>0.7957175925925926</v>
+        <v>0.9999421296296296</v>
       </c>
       <c r="U29" s="5">
-        <v>0.7309608540925266</v>
+        <v>-0.004982206405693967</v>
       </c>
       <c r="V29" s="5">
-        <v>0.1393991416309012</v>
+        <v>-0.002231759656652343</v>
       </c>
       <c r="W29" s="5">
-        <v>-0.2042824074074074</v>
+        <v>-5.787037037041642E-05</v>
       </c>
     </row>
     <row r="30" spans="1:23">
@@ -1504,22 +1504,22 @@
         <v>9</v>
       </c>
       <c r="F30" s="5">
-        <v>0.3138790035587188</v>
+        <v>0.4483985765124555</v>
       </c>
       <c r="G30" s="5">
+        <v>0.4973390557939914</v>
+      </c>
+      <c r="H30" s="5">
         <v>1</v>
       </c>
-      <c r="H30" s="5">
-        <v>0.5114004629629629</v>
-      </c>
       <c r="I30" s="5">
-        <v>-0.1110320284697509</v>
+        <v>0.000711743772241924</v>
       </c>
       <c r="J30" s="5">
-        <v>0.5392274678111588</v>
+        <v>-0.003605150214592401</v>
       </c>
       <c r="K30" s="5">
-        <v>-0.4885995370370371</v>
+        <v>0</v>
       </c>
       <c r="M30" s="4"/>
       <c r="N30" s="4"/>
@@ -1529,22 +1529,22 @@
         <v>9</v>
       </c>
       <c r="R30" s="5">
-        <v>0.4576512455516014</v>
+        <v>0.297508896797153</v>
       </c>
       <c r="S30" s="5">
-        <v>0.9430042918454935</v>
+        <v>0.3368240343347639</v>
       </c>
       <c r="T30" s="5">
-        <v>0.6142361111111111</v>
+        <v>0.9998842592592592</v>
       </c>
       <c r="U30" s="5">
-        <v>0.2377224199288256</v>
+        <v>0.009964412811387879</v>
       </c>
       <c r="V30" s="5">
-        <v>0.6065236051502145</v>
+        <v>0.006695278969957086</v>
       </c>
       <c r="W30" s="5">
-        <v>-0.3857638888888889</v>
+        <v>-0.0001157407407408328</v>
       </c>
     </row>
     <row r="39" spans="1:23">
@@ -1713,64 +1713,64 @@
         <v>1</v>
       </c>
       <c r="C43" s="4">
-        <v>0.1934763948497854</v>
+        <v>0.1998283261802575</v>
       </c>
       <c r="D43" s="4">
-        <v>0.4030092592592592</v>
+        <v>0.3678819444444444</v>
       </c>
       <c r="E43" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F43" s="5">
-        <v>0.7181494661921708</v>
+        <v>1</v>
       </c>
       <c r="G43" s="5">
-        <v>0.9994849785407725</v>
+        <v>0.1986266094420601</v>
       </c>
       <c r="H43" s="5">
-        <v>0.3368055555555555</v>
+        <v>0.3682291666666666</v>
       </c>
       <c r="I43" s="5">
-        <v>-0.2818505338078292</v>
+        <v>0</v>
       </c>
       <c r="J43" s="5">
-        <v>0.806008583690987</v>
+        <v>-0.001201716738197467</v>
       </c>
       <c r="K43" s="5">
-        <v>-0.06620370370370376</v>
+        <v>0.000347222222222221</v>
       </c>
       <c r="M43" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N43" s="4">
-        <v>0.9943060498220641</v>
+        <v>0.997153024911032</v>
       </c>
       <c r="O43" s="4">
-        <v>0.5685836909871245</v>
+        <v>0.6078969957081545</v>
       </c>
       <c r="P43" s="4">
-        <v>0.4642361111111111</v>
+        <v>0.4353009259259258</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>9</v>
       </c>
       <c r="R43" s="5">
-        <v>0.7238434163701069</v>
+        <v>0.997153024911032</v>
       </c>
       <c r="S43" s="5">
-        <v>0.9466094420600859</v>
+        <v>0.6133905579399141</v>
       </c>
       <c r="T43" s="5">
-        <v>0.4780671296296296</v>
+        <v>0.4310763888888889</v>
       </c>
       <c r="U43" s="5">
-        <v>-0.2704626334519572</v>
+        <v>0</v>
       </c>
       <c r="V43" s="5">
-        <v>0.3780257510729614</v>
+        <v>0.005493562231759674</v>
       </c>
       <c r="W43" s="5">
-        <v>0.01383101851851853</v>
+        <v>-0.004224537037036902</v>
       </c>
     </row>
     <row r="44" spans="1:23">
@@ -1782,22 +1782,22 @@
         <v>10</v>
       </c>
       <c r="F44" s="5">
-        <v>0.6405693950177935</v>
+        <v>1</v>
       </c>
       <c r="G44" s="5">
-        <v>0.4274678111587983</v>
+        <v>0.1994849785407725</v>
       </c>
       <c r="H44" s="5">
-        <v>1</v>
+        <v>0.3681712962962963</v>
       </c>
       <c r="I44" s="5">
-        <v>-0.3594306049822065</v>
+        <v>0</v>
       </c>
       <c r="J44" s="5">
-        <v>0.2339914163090129</v>
+        <v>-0.0003433476394849866</v>
       </c>
       <c r="K44" s="5">
-        <v>0.5969907407407408</v>
+        <v>0.0002893518518519156</v>
       </c>
       <c r="M44" s="4"/>
       <c r="N44" s="4"/>
@@ -1807,22 +1807,22 @@
         <v>10</v>
       </c>
       <c r="R44" s="5">
-        <v>0.4206405693950178</v>
+        <v>0.997153024911032</v>
       </c>
       <c r="S44" s="5">
-        <v>0.2945922746781116</v>
+        <v>0.6078969957081545</v>
       </c>
       <c r="T44" s="5">
-        <v>0.9999421296296296</v>
+        <v>0.4349537037037037</v>
       </c>
       <c r="U44" s="5">
-        <v>-0.5736654804270462</v>
+        <v>0</v>
       </c>
       <c r="V44" s="5">
-        <v>-0.2739914163090129</v>
+        <v>0</v>
       </c>
       <c r="W44" s="5">
-        <v>0.5357060185185185</v>
+        <v>-0.00034722222222211</v>
       </c>
     </row>
     <row r="45" spans="1:23">
@@ -1830,67 +1830,67 @@
         <v>9</v>
       </c>
       <c r="B45" s="4">
-        <v>0.3501779359430605</v>
+        <v>0.3829181494661922</v>
       </c>
       <c r="C45" s="4">
-        <v>0.9994849785407725</v>
+        <v>0.99931330472103</v>
       </c>
       <c r="D45" s="4">
-        <v>0.4594328703703703</v>
+        <v>0.4515625</v>
       </c>
       <c r="E45" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F45" s="5">
-        <v>0.9992882562277581</v>
+        <v>0.3814946619217082</v>
       </c>
       <c r="G45" s="5">
-        <v>0.2472103004291846</v>
+        <v>0.99931330472103</v>
       </c>
       <c r="H45" s="5">
-        <v>0.4780092592592594</v>
+        <v>0.4519097222222223</v>
       </c>
       <c r="I45" s="5">
-        <v>0.6491103202846975</v>
+        <v>-0.001423487544483959</v>
       </c>
       <c r="J45" s="5">
-        <v>-0.7522746781115879</v>
+        <v>0</v>
       </c>
       <c r="K45" s="5">
-        <v>0.01857638888888902</v>
+        <v>0.0003472222222222765</v>
       </c>
       <c r="M45" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N45" s="4">
-        <v>0.493950177935943</v>
+        <v>0.4085409252669039</v>
       </c>
       <c r="O45" s="4">
-        <v>0.9668669527896995</v>
+        <v>0.9618884120171675</v>
       </c>
       <c r="P45" s="4">
-        <v>0.342013888888889</v>
+        <v>0.3835069444444444</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R45" s="5">
-        <v>0.9693950177935943</v>
+        <v>0.4206405693950178</v>
       </c>
       <c r="S45" s="5">
-        <v>0.7215450643776824</v>
+        <v>0.9612017167381974</v>
       </c>
       <c r="T45" s="5">
-        <v>0.5094907407407407</v>
+        <v>0.3856481481481481</v>
       </c>
       <c r="U45" s="5">
-        <v>0.4754448398576512</v>
+        <v>0.01209964412811387</v>
       </c>
       <c r="V45" s="5">
-        <v>-0.2453218884120171</v>
+        <v>-0.0006866952789700287</v>
       </c>
       <c r="W45" s="5">
-        <v>0.1674768518518518</v>
+        <v>0.002141203703703687</v>
       </c>
     </row>
     <row r="46" spans="1:23">
@@ -1902,22 +1902,22 @@
         <v>10</v>
       </c>
       <c r="F46" s="5">
-        <v>0.405693950177936</v>
+        <v>0.3829181494661922</v>
       </c>
       <c r="G46" s="5">
-        <v>0.5641201716738198</v>
+        <v>0.99931330472103</v>
       </c>
       <c r="H46" s="5">
-        <v>1</v>
+        <v>0.451388888888889</v>
       </c>
       <c r="I46" s="5">
-        <v>0.05551601423487551</v>
+        <v>0</v>
       </c>
       <c r="J46" s="5">
-        <v>-0.4353648068669527</v>
+        <v>0</v>
       </c>
       <c r="K46" s="5">
-        <v>0.5405671296296297</v>
+        <v>-0.0001736111111110272</v>
       </c>
       <c r="M46" s="4"/>
       <c r="N46" s="4"/>
@@ -1927,22 +1927,22 @@
         <v>10</v>
       </c>
       <c r="R46" s="5">
-        <v>0.2476868327402135</v>
+        <v>0.4071174377224199</v>
       </c>
       <c r="S46" s="5">
-        <v>0.3563948497854078</v>
+        <v>0.961716738197425</v>
       </c>
       <c r="T46" s="5">
-        <v>0.9999421296296296</v>
+        <v>0.385474537037037</v>
       </c>
       <c r="U46" s="5">
-        <v>-0.2462633451957295</v>
+        <v>-0.001423487544483959</v>
       </c>
       <c r="V46" s="5">
-        <v>-0.6104721030042917</v>
+        <v>-0.0001716738197424794</v>
       </c>
       <c r="W46" s="5">
-        <v>0.6579282407407406</v>
+        <v>0.001967592592592604</v>
       </c>
     </row>
     <row r="47" spans="1:23">
@@ -1950,10 +1950,10 @@
         <v>10</v>
       </c>
       <c r="B47" s="4">
-        <v>0.4526690391459075</v>
+        <v>0.4405693950177936</v>
       </c>
       <c r="C47" s="4">
-        <v>0.4863519313304721</v>
+        <v>0.5040343347639485</v>
       </c>
       <c r="D47" s="4">
         <v>1</v>
@@ -1962,55 +1962,55 @@
         <v>8</v>
       </c>
       <c r="F47" s="5">
-        <v>0.995017793594306</v>
+        <v>0.4405693950177936</v>
       </c>
       <c r="G47" s="5">
-        <v>0.2836051502145923</v>
+        <v>0.5042060085836909</v>
       </c>
       <c r="H47" s="5">
-        <v>0.6358217592592592</v>
+        <v>1</v>
       </c>
       <c r="I47" s="5">
-        <v>0.5423487544483985</v>
+        <v>0</v>
       </c>
       <c r="J47" s="5">
-        <v>-0.2027467811158798</v>
+        <v>0.0001716738197423684</v>
       </c>
       <c r="K47" s="5">
-        <v>-0.3641782407407408</v>
+        <v>0</v>
       </c>
       <c r="M47" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N47" s="4">
-        <v>0.2106761565836299</v>
+        <v>0.2427046263345196</v>
       </c>
       <c r="O47" s="4">
-        <v>0.3230901287553648</v>
+        <v>0.2894420600858369</v>
       </c>
       <c r="P47" s="4">
+        <v>1</v>
+      </c>
+      <c r="Q47" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="R47" s="5">
+        <v>0.2533807829181495</v>
+      </c>
+      <c r="S47" s="5">
+        <v>0.2939055793991416</v>
+      </c>
+      <c r="T47" s="5">
         <v>0.9999421296296296</v>
       </c>
-      <c r="Q47" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="R47" s="5">
-        <v>0.9430604982206405</v>
-      </c>
-      <c r="S47" s="5">
-        <v>0.4106437768240343</v>
-      </c>
-      <c r="T47" s="5">
-        <v>0.8483217592592591</v>
-      </c>
       <c r="U47" s="5">
-        <v>0.7323843416370106</v>
+        <v>0.01067615658362991</v>
       </c>
       <c r="V47" s="5">
-        <v>0.0875536480686695</v>
+        <v>0.004463519313304687</v>
       </c>
       <c r="W47" s="5">
-        <v>-0.1516203703703705</v>
+        <v>-5.787037037041642E-05</v>
       </c>
     </row>
     <row r="48" spans="1:23">
@@ -2022,22 +2022,22 @@
         <v>9</v>
       </c>
       <c r="F48" s="5">
-        <v>0.3822064056939501</v>
+        <v>0.4391459074733096</v>
       </c>
       <c r="G48" s="5">
-        <v>0.999656652360515</v>
+        <v>0.5062660944206009</v>
       </c>
       <c r="H48" s="5">
-        <v>0.5244212962962962</v>
+        <v>1</v>
       </c>
       <c r="I48" s="5">
-        <v>-0.07046263345195736</v>
+        <v>-0.001423487544484014</v>
       </c>
       <c r="J48" s="5">
-        <v>0.513304721030043</v>
+        <v>0.002231759656652343</v>
       </c>
       <c r="K48" s="5">
-        <v>-0.4755787037037038</v>
+        <v>0</v>
       </c>
       <c r="M48" s="4"/>
       <c r="N48" s="4"/>
@@ -2047,22 +2047,22 @@
         <v>9</v>
       </c>
       <c r="R48" s="5">
-        <v>0.3871886120996441</v>
+        <v>0.2427046263345196</v>
       </c>
       <c r="S48" s="5">
-        <v>0.9404291845493562</v>
+        <v>0.2923605150214593</v>
       </c>
       <c r="T48" s="5">
-        <v>0.672974537037037</v>
+        <v>1</v>
       </c>
       <c r="U48" s="5">
-        <v>0.1765124555160142</v>
+        <v>0</v>
       </c>
       <c r="V48" s="5">
-        <v>0.6173390557939914</v>
+        <v>0.002918454935622317</v>
       </c>
       <c r="W48" s="5">
-        <v>-0.3269675925925926</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:23">
@@ -2231,31 +2231,31 @@
         <v>1</v>
       </c>
       <c r="C61" s="4">
-        <v>0.2466952789699571</v>
+        <v>0.288412017167382</v>
       </c>
       <c r="D61" s="4">
-        <v>0.4410300925925926</v>
+        <v>0.436863425925926</v>
       </c>
       <c r="E61" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F61" s="5">
-        <v>0.9281138790035588</v>
+        <v>0.6035587188612099</v>
       </c>
       <c r="G61" s="5">
-        <v>1</v>
+        <v>0.4825751072961373</v>
       </c>
       <c r="H61" s="5">
-        <v>0.38125</v>
+        <v>0.2628472222222222</v>
       </c>
       <c r="I61" s="5">
-        <v>-0.07188612099644121</v>
+        <v>-0.3964412811387901</v>
       </c>
       <c r="J61" s="5">
-        <v>0.753304721030043</v>
+        <v>0.1941630901287553</v>
       </c>
       <c r="K61" s="5">
-        <v>-0.05978009259259265</v>
+        <v>-0.1740162037037038</v>
       </c>
       <c r="M61" s="4" t="s">
         <v>8</v>
@@ -2264,31 +2264,31 @@
         <v>1</v>
       </c>
       <c r="O61" s="4">
-        <v>0.2096137339055794</v>
+        <v>0.2223175965665236</v>
       </c>
       <c r="P61" s="4">
-        <v>0.4032986111111111</v>
+        <v>0.447800925925926</v>
       </c>
       <c r="Q61" s="5" t="s">
         <v>9</v>
       </c>
       <c r="R61" s="5">
-        <v>0.8925266903914592</v>
+        <v>0.3758007117437723</v>
       </c>
       <c r="S61" s="5">
-        <v>1</v>
+        <v>0.2417167381974249</v>
       </c>
       <c r="T61" s="5">
-        <v>0.2612847222222222</v>
+        <v>0.3390625</v>
       </c>
       <c r="U61" s="5">
-        <v>-0.1074733096085408</v>
+        <v>-0.6241992882562277</v>
       </c>
       <c r="V61" s="5">
-        <v>0.7903862660944205</v>
+        <v>0.01939914163090126</v>
       </c>
       <c r="W61" s="5">
-        <v>-0.1420138888888889</v>
+        <v>-0.108738425925926</v>
       </c>
     </row>
     <row r="62" spans="1:23">
@@ -2300,22 +2300,22 @@
         <v>10</v>
       </c>
       <c r="F62" s="5">
-        <v>0.9864768683274022</v>
+        <v>0.494661921708185</v>
       </c>
       <c r="G62" s="5">
-        <v>0.4721030042918454</v>
+        <v>0.1854077253218884</v>
       </c>
       <c r="H62" s="5">
-        <v>1</v>
+        <v>0.4465277777777777</v>
       </c>
       <c r="I62" s="5">
-        <v>-0.01352313167259778</v>
+        <v>-0.505338078291815</v>
       </c>
       <c r="J62" s="5">
-        <v>0.2254077253218884</v>
+        <v>-0.1030042918454936</v>
       </c>
       <c r="K62" s="5">
-        <v>0.5589699074074074</v>
+        <v>0.009664351851851771</v>
       </c>
       <c r="M62" s="4"/>
       <c r="N62" s="4"/>
@@ -2325,22 +2325,22 @@
         <v>10</v>
       </c>
       <c r="R62" s="5">
-        <v>0.9138790035587189</v>
+        <v>0.4839857651245551</v>
       </c>
       <c r="S62" s="5">
-        <v>0.3476394849785408</v>
+        <v>0.2717596566523605</v>
       </c>
       <c r="T62" s="5">
-        <v>1</v>
+        <v>0.4920138888888889</v>
       </c>
       <c r="U62" s="5">
-        <v>-0.08612099644128113</v>
+        <v>-0.5160142348754448</v>
       </c>
       <c r="V62" s="5">
-        <v>0.1380257510729614</v>
+        <v>0.0494420600858369</v>
       </c>
       <c r="W62" s="5">
-        <v>0.5967013888888888</v>
+        <v>0.04421296296296295</v>
       </c>
     </row>
     <row r="63" spans="1:23">
@@ -2348,67 +2348,67 @@
         <v>9</v>
       </c>
       <c r="B63" s="4">
-        <v>0.2811387900355872</v>
+        <v>0.2206405693950178</v>
       </c>
       <c r="C63" s="4">
         <v>1</v>
       </c>
       <c r="D63" s="4">
-        <v>0.330787037037037</v>
+        <v>0.358738425925926</v>
       </c>
       <c r="E63" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F63" s="5">
-        <v>1</v>
+        <v>0.2277580071174377</v>
       </c>
       <c r="G63" s="5">
-        <v>0.4920171673819743</v>
+        <v>0.8846351931330473</v>
       </c>
       <c r="H63" s="5">
-        <v>0.4060185185185185</v>
+        <v>0.3291666666666667</v>
       </c>
       <c r="I63" s="5">
-        <v>0.7188612099644127</v>
+        <v>0.007117437722419906</v>
       </c>
       <c r="J63" s="5">
-        <v>-0.5079828326180257</v>
+        <v>-0.1153648068669527</v>
       </c>
       <c r="K63" s="5">
-        <v>0.07523148148148145</v>
+        <v>-0.02957175925925931</v>
       </c>
       <c r="M63" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N63" s="4">
-        <v>0.4476868327402135</v>
+        <v>0.5096085409252669</v>
       </c>
       <c r="O63" s="4">
         <v>1</v>
       </c>
       <c r="P63" s="4">
-        <v>0.2438078703703704</v>
+        <v>0.2461805555555555</v>
       </c>
       <c r="Q63" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R63" s="5">
-        <v>0.99644128113879</v>
+        <v>0.5516014234875445</v>
       </c>
       <c r="S63" s="5">
-        <v>0.9699570815450643</v>
+        <v>0.7654935622317597</v>
       </c>
       <c r="T63" s="5">
-        <v>0.2331018518518519</v>
+        <v>0.2220486111111111</v>
       </c>
       <c r="U63" s="5">
-        <v>0.5487544483985765</v>
+        <v>0.04199288256227762</v>
       </c>
       <c r="V63" s="5">
-        <v>-0.03004291845493567</v>
+        <v>-0.2345064377682403</v>
       </c>
       <c r="W63" s="5">
-        <v>-0.01070601851851855</v>
+        <v>-0.02413194444444441</v>
       </c>
     </row>
     <row r="64" spans="1:23">
@@ -2420,22 +2420,22 @@
         <v>10</v>
       </c>
       <c r="F64" s="5">
-        <v>0.3622775800711744</v>
+        <v>0.1736654804270463</v>
       </c>
       <c r="G64" s="5">
-        <v>0.9859227467811159</v>
+        <v>0.774763948497854</v>
       </c>
       <c r="H64" s="5">
-        <v>1</v>
+        <v>0.3367476851851852</v>
       </c>
       <c r="I64" s="5">
-        <v>0.08113879003558716</v>
+        <v>-0.04697508896797153</v>
       </c>
       <c r="J64" s="5">
-        <v>-0.01407725321888409</v>
+        <v>-0.225236051502146</v>
       </c>
       <c r="K64" s="5">
-        <v>0.669212962962963</v>
+        <v>-0.02199074074074076</v>
       </c>
       <c r="M64" s="4"/>
       <c r="N64" s="4"/>
@@ -2445,22 +2445,22 @@
         <v>10</v>
       </c>
       <c r="R64" s="5">
-        <v>0.2</v>
+        <v>0.5131672597864768</v>
       </c>
       <c r="S64" s="5">
-        <v>0.559656652360515</v>
+        <v>0.5881545064377682</v>
       </c>
       <c r="T64" s="5">
-        <v>1</v>
+        <v>0.2364583333333334</v>
       </c>
       <c r="U64" s="5">
-        <v>-0.2476868327402135</v>
+        <v>0.003558718861209953</v>
       </c>
       <c r="V64" s="5">
-        <v>-0.440343347639485</v>
+        <v>-0.4118454935622318</v>
       </c>
       <c r="W64" s="5">
-        <v>0.7561921296296296</v>
+        <v>-0.009722222222222188</v>
       </c>
     </row>
     <row r="65" spans="1:23">
@@ -2468,10 +2468,10 @@
         <v>10</v>
       </c>
       <c r="B65" s="4">
-        <v>0.3174377224199288</v>
+        <v>0.3295373665480427</v>
       </c>
       <c r="C65" s="4">
-        <v>0.423175965665236</v>
+        <v>0.4520171673819743</v>
       </c>
       <c r="D65" s="4">
         <v>1</v>
@@ -2480,31 +2480,31 @@
         <v>8</v>
       </c>
       <c r="F65" s="5">
-        <v>1</v>
+        <v>0.3508896797153025</v>
       </c>
       <c r="G65" s="5">
-        <v>0.1946781115879828</v>
+        <v>0.552274678111588</v>
       </c>
       <c r="H65" s="5">
-        <v>0.9972222222222221</v>
+        <v>0.771875</v>
       </c>
       <c r="I65" s="5">
-        <v>0.6825622775800712</v>
+        <v>0.02135231316725988</v>
       </c>
       <c r="J65" s="5">
-        <v>-0.2284978540772532</v>
+        <v>0.1002575107296138</v>
       </c>
       <c r="K65" s="5">
-        <v>-0.002777777777777879</v>
+        <v>-0.228125</v>
       </c>
       <c r="M65" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N65" s="4">
-        <v>0.1644128113879004</v>
+        <v>0.1615658362989324</v>
       </c>
       <c r="O65" s="4">
-        <v>0.2453218884120171</v>
+        <v>0.2415450643776824</v>
       </c>
       <c r="P65" s="4">
         <v>1</v>
@@ -2513,22 +2513,22 @@
         <v>8</v>
       </c>
       <c r="R65" s="5">
+        <v>0.1615658362989324</v>
+      </c>
+      <c r="S65" s="5">
+        <v>0.2410300429184549</v>
+      </c>
+      <c r="T65" s="5">
         <v>1</v>
       </c>
-      <c r="S65" s="5">
-        <v>0.2520171673819743</v>
-      </c>
-      <c r="T65" s="5">
-        <v>0.8545138888888889</v>
-      </c>
       <c r="U65" s="5">
-        <v>0.8355871886120996</v>
+        <v>0</v>
       </c>
       <c r="V65" s="5">
-        <v>0.006695278969957141</v>
+        <v>-0.0005150214592274938</v>
       </c>
       <c r="W65" s="5">
-        <v>-0.1454861111111111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:23">
@@ -2540,22 +2540,22 @@
         <v>9</v>
       </c>
       <c r="F66" s="5">
-        <v>0.3124555160142349</v>
+        <v>0.3160142348754448</v>
       </c>
       <c r="G66" s="5">
-        <v>1</v>
+        <v>0.4449785407725322</v>
       </c>
       <c r="H66" s="5">
-        <v>0.999363425925926</v>
+        <v>0.9046296296296298</v>
       </c>
       <c r="I66" s="5">
-        <v>-0.004982206405693967</v>
+        <v>-0.01352313167259783</v>
       </c>
       <c r="J66" s="5">
-        <v>0.5768240343347639</v>
+        <v>-0.007038626609442045</v>
       </c>
       <c r="K66" s="5">
-        <v>-0.0006365740740740256</v>
+        <v>-0.09537037037037022</v>
       </c>
       <c r="M66" s="4"/>
       <c r="N66" s="4"/>
@@ -2565,22 +2565,22 @@
         <v>9</v>
       </c>
       <c r="R66" s="5">
-        <v>0.5572953736654804</v>
+        <v>0.1615658362989324</v>
       </c>
       <c r="S66" s="5">
+        <v>0.2413733905579399</v>
+      </c>
+      <c r="T66" s="5">
         <v>1</v>
       </c>
-      <c r="T66" s="5">
-        <v>0.7630787037037037</v>
-      </c>
       <c r="U66" s="5">
-        <v>0.3928825622775801</v>
+        <v>0</v>
       </c>
       <c r="V66" s="5">
-        <v>0.7546781115879828</v>
+        <v>-0.0001716738197425072</v>
       </c>
       <c r="W66" s="5">
-        <v>-0.2369212962962963</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:23">
@@ -2746,34 +2746,34 @@
         <v>8</v>
       </c>
       <c r="B79" s="4">
-        <v>0.9814946619217082</v>
+        <v>0.9750889679715302</v>
       </c>
       <c r="C79" s="4">
-        <v>0.3895278969957081</v>
+        <v>0.3879828326180257</v>
       </c>
       <c r="D79" s="4">
-        <v>0.3936921296296297</v>
+        <v>0.3759259259259259</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F79" s="5">
-        <v>0.9209964412811388</v>
+        <v>0.9701067615658363</v>
       </c>
       <c r="G79" s="5">
-        <v>0.9991416309012875</v>
+        <v>0.4080686695278971</v>
       </c>
       <c r="H79" s="5">
-        <v>0.4355902777777778</v>
+        <v>0.4592013888888888</v>
       </c>
       <c r="I79" s="5">
-        <v>-0.06049822064056942</v>
+        <v>-0.004982206405693912</v>
       </c>
       <c r="J79" s="5">
-        <v>0.6096137339055794</v>
+        <v>0.02008583690987131</v>
       </c>
       <c r="K79" s="5">
-        <v>0.04189814814814807</v>
+        <v>0.08327546296296295</v>
       </c>
       <c r="M79" s="4" t="s">
         <v>8</v>
@@ -2782,31 +2782,31 @@
         <v>1</v>
       </c>
       <c r="O79" s="4">
-        <v>0.2478969957081545</v>
+        <v>0.2566523605150214</v>
       </c>
       <c r="P79" s="4">
-        <v>0.3895833333333333</v>
+        <v>0.3605902777777777</v>
       </c>
       <c r="Q79" s="5" t="s">
         <v>9</v>
       </c>
       <c r="R79" s="5">
-        <v>0.9551601423487543</v>
+        <v>1</v>
       </c>
       <c r="S79" s="5">
-        <v>0.9945064377682403</v>
+        <v>0.2520171673819743</v>
       </c>
       <c r="T79" s="5">
-        <v>0.3157986111111111</v>
+        <v>0.3596643518518519</v>
       </c>
       <c r="U79" s="5">
-        <v>-0.04483985765124565</v>
+        <v>0</v>
       </c>
       <c r="V79" s="5">
-        <v>0.7466094420600858</v>
+        <v>-0.004635193133047166</v>
       </c>
       <c r="W79" s="5">
-        <v>-0.07378472222222215</v>
+        <v>-0.0009259259259258856</v>
       </c>
     </row>
     <row r="80" spans="1:23">
@@ -2818,22 +2818,22 @@
         <v>10</v>
       </c>
       <c r="F80" s="5">
-        <v>0.9608540925266904</v>
+        <v>0.9758007117437721</v>
       </c>
       <c r="G80" s="5">
-        <v>0.3400858369098713</v>
+        <v>0.4089270386266095</v>
       </c>
       <c r="H80" s="5">
-        <v>1</v>
+        <v>0.3614583333333333</v>
       </c>
       <c r="I80" s="5">
-        <v>-0.02064056939501779</v>
+        <v>0.000711743772241924</v>
       </c>
       <c r="J80" s="5">
-        <v>-0.04944206008583685</v>
+        <v>0.02094420600858371</v>
       </c>
       <c r="K80" s="5">
-        <v>0.6063078703703704</v>
+        <v>-0.01446759259259256</v>
       </c>
       <c r="M80" s="4"/>
       <c r="N80" s="4"/>
@@ -2843,22 +2843,22 @@
         <v>10</v>
       </c>
       <c r="R80" s="5">
-        <v>0.9608540925266904</v>
+        <v>0.8597864768683274</v>
       </c>
       <c r="S80" s="5">
-        <v>0.2506437768240343</v>
+        <v>0.2357081545064378</v>
       </c>
       <c r="T80" s="5">
-        <v>1</v>
+        <v>0.3340277777777777</v>
       </c>
       <c r="U80" s="5">
-        <v>-0.03914590747330959</v>
+        <v>-0.1402135231316726</v>
       </c>
       <c r="V80" s="5">
-        <v>0.002746781115879837</v>
+        <v>-0.02094420600858368</v>
       </c>
       <c r="W80" s="5">
-        <v>0.6104166666666667</v>
+        <v>-0.02656250000000004</v>
       </c>
     </row>
     <row r="81" spans="1:23">
@@ -2866,67 +2866,67 @@
         <v>9</v>
       </c>
       <c r="B81" s="4">
-        <v>0.6526690391459075</v>
+        <v>0.6839857651245551</v>
       </c>
       <c r="C81" s="4">
-        <v>0.99931330472103</v>
+        <v>0.9998283261802575</v>
       </c>
       <c r="D81" s="4">
-        <v>0.3485532407407408</v>
+        <v>0.3414351851851852</v>
       </c>
       <c r="E81" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F81" s="5">
-        <v>0.9758007117437723</v>
+        <v>0.7402135231316727</v>
       </c>
       <c r="G81" s="5">
-        <v>0.8281545064377681</v>
+        <v>0.9879828326180258</v>
       </c>
       <c r="H81" s="5">
-        <v>0.3501157407407408</v>
+        <v>0.3532407407407407</v>
       </c>
       <c r="I81" s="5">
-        <v>0.3231316725978648</v>
+        <v>0.05622775800711755</v>
       </c>
       <c r="J81" s="5">
-        <v>-0.1711587982832619</v>
+        <v>-0.01184549356223175</v>
       </c>
       <c r="K81" s="5">
-        <v>0.001562499999999967</v>
+        <v>0.01180555555555557</v>
       </c>
       <c r="M81" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N81" s="4">
-        <v>0.5544483985765124</v>
+        <v>0.5565836298932385</v>
       </c>
       <c r="O81" s="4">
-        <v>0.9945064377682403</v>
+        <v>0.9972532188841201</v>
       </c>
       <c r="P81" s="4">
-        <v>0.4028356481481481</v>
+        <v>0.3375</v>
       </c>
       <c r="Q81" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R81" s="5">
-        <v>1</v>
+        <v>0.5786476868327401</v>
       </c>
       <c r="S81" s="5">
-        <v>0.6559656652360515</v>
+        <v>0.9339055793991416</v>
       </c>
       <c r="T81" s="5">
-        <v>0.3669560185185185</v>
+        <v>0.2935763888888889</v>
       </c>
       <c r="U81" s="5">
-        <v>0.4455516014234876</v>
+        <v>0.02206405693950164</v>
       </c>
       <c r="V81" s="5">
-        <v>-0.3385407725321888</v>
+        <v>-0.06334763948497846</v>
       </c>
       <c r="W81" s="5">
-        <v>-0.03587962962962959</v>
+        <v>-0.04392361111111109</v>
       </c>
     </row>
     <row r="82" spans="1:23">
@@ -2938,22 +2938,22 @@
         <v>10</v>
       </c>
       <c r="F82" s="5">
-        <v>0.6604982206405693</v>
+        <v>0.6790035587188612</v>
       </c>
       <c r="G82" s="5">
-        <v>0.9639484978540771</v>
+        <v>0.967381974248927</v>
       </c>
       <c r="H82" s="5">
-        <v>1</v>
+        <v>0.3384837962962963</v>
       </c>
       <c r="I82" s="5">
-        <v>0.00782918149466183</v>
+        <v>-0.004982206405693912</v>
       </c>
       <c r="J82" s="5">
-        <v>-0.03536480686695287</v>
+        <v>-0.0324463519313305</v>
       </c>
       <c r="K82" s="5">
-        <v>0.6514467592592592</v>
+        <v>-0.002951388888888906</v>
       </c>
       <c r="M82" s="4"/>
       <c r="N82" s="4"/>
@@ -2963,22 +2963,22 @@
         <v>10</v>
       </c>
       <c r="R82" s="5">
-        <v>0.197864768683274</v>
+        <v>0.5658362989323844</v>
       </c>
       <c r="S82" s="5">
-        <v>0.3205150214592274</v>
+        <v>0.9339055793991416</v>
       </c>
       <c r="T82" s="5">
-        <v>1</v>
+        <v>0.3556134259259259</v>
       </c>
       <c r="U82" s="5">
-        <v>-0.3565836298932384</v>
+        <v>0.0092526690391459</v>
       </c>
       <c r="V82" s="5">
-        <v>-0.6739914163090128</v>
+        <v>-0.06334763948497846</v>
       </c>
       <c r="W82" s="5">
-        <v>0.5971643518518519</v>
+        <v>0.01811342592592591</v>
       </c>
     </row>
     <row r="83" spans="1:23">
@@ -2986,10 +2986,10 @@
         <v>10</v>
       </c>
       <c r="B83" s="4">
-        <v>0.5252669039145907</v>
+        <v>0.601423487544484</v>
       </c>
       <c r="C83" s="4">
-        <v>0.2812017167381974</v>
+        <v>0.3327038626609442</v>
       </c>
       <c r="D83" s="4">
         <v>1</v>
@@ -2998,31 +2998,31 @@
         <v>8</v>
       </c>
       <c r="F83" s="5">
-        <v>0.9807829181494661</v>
+        <v>0.698220640569395</v>
       </c>
       <c r="G83" s="5">
-        <v>0.4552789699570816</v>
+        <v>0.3332188841201716</v>
       </c>
       <c r="H83" s="5">
-        <v>0.6148148148148149</v>
+        <v>0.999826388888889</v>
       </c>
       <c r="I83" s="5">
-        <v>0.4555160142348753</v>
+        <v>0.09679715302491099</v>
       </c>
       <c r="J83" s="5">
-        <v>0.1740772532188842</v>
+        <v>0.0005150214592274382</v>
       </c>
       <c r="K83" s="5">
-        <v>-0.3851851851851851</v>
+        <v>-0.0001736111111110272</v>
       </c>
       <c r="M83" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N83" s="4">
-        <v>0.1750889679715302</v>
+        <v>0.1679715302491103</v>
       </c>
       <c r="O83" s="4">
-        <v>0.2669527896995708</v>
+        <v>0.2624892703862661</v>
       </c>
       <c r="P83" s="4">
         <v>1</v>
@@ -3031,22 +3031,22 @@
         <v>8</v>
       </c>
       <c r="R83" s="5">
+        <v>0.1679715302491103</v>
+      </c>
+      <c r="S83" s="5">
+        <v>0.2624892703862661</v>
+      </c>
+      <c r="T83" s="5">
         <v>1</v>
       </c>
-      <c r="S83" s="5">
-        <v>0.2990557939914163</v>
-      </c>
-      <c r="T83" s="5">
-        <v>0.9545717592592593</v>
-      </c>
       <c r="U83" s="5">
-        <v>0.8249110320284698</v>
+        <v>0</v>
       </c>
       <c r="V83" s="5">
-        <v>0.03210300429184548</v>
+        <v>0</v>
       </c>
       <c r="W83" s="5">
-        <v>-0.0454282407407407</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:23">
@@ -3058,22 +3058,22 @@
         <v>9</v>
       </c>
       <c r="F84" s="5">
-        <v>0.7572953736654804</v>
+        <v>0.5039145907473309</v>
       </c>
       <c r="G84" s="5">
-        <v>0.99931330472103</v>
+        <v>0.3230901287553648</v>
       </c>
       <c r="H84" s="5">
-        <v>0.928587962962963</v>
+        <v>1</v>
       </c>
       <c r="I84" s="5">
-        <v>0.2320284697508896</v>
+        <v>-0.09750889679715313</v>
       </c>
       <c r="J84" s="5">
-        <v>0.7181115879828326</v>
+        <v>-0.009613733905579402</v>
       </c>
       <c r="K84" s="5">
-        <v>-0.07141203703703702</v>
+        <v>0</v>
       </c>
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
@@ -3083,22 +3083,22 @@
         <v>9</v>
       </c>
       <c r="R84" s="5">
-        <v>0.5601423487544483</v>
+        <v>0.1679715302491103</v>
       </c>
       <c r="S84" s="5">
-        <v>0.9953648068669528</v>
+        <v>0.2624892703862661</v>
       </c>
       <c r="T84" s="5">
-        <v>0.5623842592592593</v>
+        <v>0.8550925925925925</v>
       </c>
       <c r="U84" s="5">
-        <v>0.3850533807829181</v>
+        <v>0</v>
       </c>
       <c r="V84" s="5">
-        <v>0.728412017167382</v>
+        <v>0</v>
       </c>
       <c r="W84" s="5">
-        <v>-0.4376157407407407</v>
+        <v>-0.1449074074074075</v>
       </c>
     </row>
     <row r="93" spans="1:23">
@@ -3264,67 +3264,67 @@
         <v>8</v>
       </c>
       <c r="B97" s="4">
-        <v>0.9544483985765124</v>
+        <v>0.9651245551601424</v>
       </c>
       <c r="C97" s="4">
-        <v>0.2777682403433476</v>
+        <v>0.271931330472103</v>
       </c>
       <c r="D97" s="4">
-        <v>0.4100115740740741</v>
+        <v>0.4488425925925926</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>9</v>
       </c>
       <c r="F97" s="5">
-        <v>0.6562277580071176</v>
+        <v>0.7743772241992883</v>
       </c>
       <c r="G97" s="5">
-        <v>0.9788841201716739</v>
+        <v>0.2609442060085837</v>
       </c>
       <c r="H97" s="5">
-        <v>0.5777199074074074</v>
+        <v>0.4305555555555555</v>
       </c>
       <c r="I97" s="5">
-        <v>-0.2982206405693948</v>
+        <v>-0.1907473309608541</v>
       </c>
       <c r="J97" s="5">
-        <v>0.7011158798283263</v>
+        <v>-0.01098712446351929</v>
       </c>
       <c r="K97" s="5">
-        <v>0.1677083333333333</v>
+        <v>-0.0182870370370371</v>
       </c>
       <c r="M97" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N97" s="4">
+        <v>0.9487544483985765</v>
+      </c>
+      <c r="O97" s="4">
+        <v>0.3272103004291845</v>
+      </c>
+      <c r="P97" s="4">
+        <v>0.3472222222222222</v>
+      </c>
+      <c r="Q97" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="R97" s="5">
         <v>0.9480427046263346</v>
       </c>
-      <c r="O97" s="4">
-        <v>0.3275536480686695</v>
-      </c>
-      <c r="P97" s="4">
-        <v>0.3443287037037037</v>
-      </c>
-      <c r="Q97" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="R97" s="5">
-        <v>0.9430604982206405</v>
-      </c>
       <c r="S97" s="5">
-        <v>0.8051502145922746</v>
+        <v>0.3270386266094421</v>
       </c>
       <c r="T97" s="5">
-        <v>0.2782986111111111</v>
+        <v>0.3475694444444445</v>
       </c>
       <c r="U97" s="5">
-        <v>-0.004982206405694023</v>
+        <v>-0.000711743772241924</v>
       </c>
       <c r="V97" s="5">
-        <v>0.4775965665236051</v>
+        <v>-0.0001716738197424794</v>
       </c>
       <c r="W97" s="5">
-        <v>-0.06603009259259263</v>
+        <v>0.0003472222222222765</v>
       </c>
     </row>
     <row r="98" spans="1:23">
@@ -3336,22 +3336,22 @@
         <v>10</v>
       </c>
       <c r="F98" s="5">
-        <v>0.7850533807829182</v>
+        <v>0.7302491103202846</v>
       </c>
       <c r="G98" s="5">
-        <v>0.2774248927038626</v>
+        <v>0.1933047210300429</v>
       </c>
       <c r="H98" s="5">
-        <v>0.999826388888889</v>
+        <v>0.427025462962963</v>
       </c>
       <c r="I98" s="5">
-        <v>-0.1693950177935942</v>
+        <v>-0.2348754448398578</v>
       </c>
       <c r="J98" s="5">
-        <v>-0.0003433476394850143</v>
+        <v>-0.07862660944206007</v>
       </c>
       <c r="K98" s="5">
-        <v>0.5898148148148149</v>
+        <v>-0.02181712962962967</v>
       </c>
       <c r="M98" s="4"/>
       <c r="N98" s="4"/>
@@ -3361,22 +3361,22 @@
         <v>10</v>
       </c>
       <c r="R98" s="5">
-        <v>0.6590747330960854</v>
+        <v>0.9480427046263346</v>
       </c>
       <c r="S98" s="5">
-        <v>0.279656652360515</v>
+        <v>0.3272103004291845</v>
       </c>
       <c r="T98" s="5">
-        <v>0.9788773148148149</v>
+        <v>0.3473958333333333</v>
       </c>
       <c r="U98" s="5">
-        <v>-0.2889679715302491</v>
+        <v>-0.000711743772241924</v>
       </c>
       <c r="V98" s="5">
-        <v>-0.04789699570815453</v>
+        <v>0</v>
       </c>
       <c r="W98" s="5">
-        <v>0.6345486111111112</v>
+        <v>0.0001736111111110827</v>
       </c>
     </row>
     <row r="99" spans="1:23">
@@ -3384,67 +3384,67 @@
         <v>9</v>
       </c>
       <c r="B99" s="4">
-        <v>0.303914590747331</v>
+        <v>0.2604982206405694</v>
       </c>
       <c r="C99" s="4">
-        <v>0.979570815450644</v>
+        <v>0.9783690987124464</v>
       </c>
       <c r="D99" s="4">
-        <v>0.3870949074074074</v>
+        <v>0.3795138888888889</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F99" s="5">
-        <v>0.904626334519573</v>
+        <v>0.3430604982206406</v>
       </c>
       <c r="G99" s="5">
-        <v>0.7987982832618025</v>
+        <v>0.9409442060085838</v>
       </c>
       <c r="H99" s="5">
-        <v>0.4126736111111111</v>
+        <v>0.4109953703703703</v>
       </c>
       <c r="I99" s="5">
-        <v>0.600711743772242</v>
+        <v>0.08256227758007118</v>
       </c>
       <c r="J99" s="5">
-        <v>-0.1807725321888415</v>
+        <v>-0.03742489270386262</v>
       </c>
       <c r="K99" s="5">
-        <v>0.02557870370370363</v>
+        <v>0.03148148148148144</v>
       </c>
       <c r="M99" s="4" t="s">
         <v>9</v>
       </c>
       <c r="N99" s="4">
-        <v>0.398576512455516</v>
+        <v>0.4512455516014235</v>
       </c>
       <c r="O99" s="4">
-        <v>0.9884978540772533</v>
+        <v>0.9919313304721029</v>
       </c>
       <c r="P99" s="4">
-        <v>0.4182291666666667</v>
+        <v>0.3975115740740741</v>
       </c>
       <c r="Q99" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R99" s="5">
-        <v>0.8982206405693949</v>
+        <v>0.4334519572953737</v>
       </c>
       <c r="S99" s="5">
-        <v>0.6090987124463518</v>
+        <v>0.8846351931330471</v>
       </c>
       <c r="T99" s="5">
-        <v>0.5179976851851851</v>
+        <v>0.3960648148148148</v>
       </c>
       <c r="U99" s="5">
-        <v>0.4996441281138789</v>
+        <v>-0.01779359430604976</v>
       </c>
       <c r="V99" s="5">
-        <v>-0.3793991416309015</v>
+        <v>-0.1072961373390559</v>
       </c>
       <c r="W99" s="5">
-        <v>0.09976851851851837</v>
+        <v>-0.001446759259259245</v>
       </c>
     </row>
     <row r="100" spans="1:23">
@@ -3456,22 +3456,22 @@
         <v>10</v>
       </c>
       <c r="F100" s="5">
-        <v>0.2455516014234876</v>
+        <v>0.3096085409252669</v>
       </c>
       <c r="G100" s="5">
-        <v>0.5541630901287553</v>
+        <v>0.7720171673819742</v>
       </c>
       <c r="H100" s="5">
-        <v>0.9996527777777777</v>
+        <v>0.4036458333333334</v>
       </c>
       <c r="I100" s="5">
-        <v>-0.05836298932384337</v>
+        <v>0.04911032028469753</v>
       </c>
       <c r="J100" s="5">
-        <v>-0.4254077253218886</v>
+        <v>-0.2063519313304721</v>
       </c>
       <c r="K100" s="5">
-        <v>0.6125578703703702</v>
+        <v>0.0241319444444445</v>
       </c>
       <c r="M100" s="4"/>
       <c r="N100" s="4"/>
@@ -3481,22 +3481,22 @@
         <v>10</v>
       </c>
       <c r="R100" s="5">
-        <v>0.4918149466192171</v>
+        <v>0.4498220640569395</v>
       </c>
       <c r="S100" s="5">
-        <v>0.5074678111587982</v>
+        <v>0.7654935622317597</v>
       </c>
       <c r="T100" s="5">
-        <v>0.9988425925925926</v>
+        <v>0.4012731481481482</v>
       </c>
       <c r="U100" s="5">
-        <v>0.09323843416370109</v>
+        <v>-0.001423487544484014</v>
       </c>
       <c r="V100" s="5">
-        <v>-0.4810300429184551</v>
+        <v>-0.2264377682403432</v>
       </c>
       <c r="W100" s="5">
-        <v>0.5806134259259259</v>
+        <v>0.003761574074074125</v>
       </c>
     </row>
     <row r="101" spans="1:23">
@@ -3504,67 +3504,67 @@
         <v>10</v>
       </c>
       <c r="B101" s="4">
-        <v>0.3558718861209965</v>
+        <v>0.306049822064057</v>
       </c>
       <c r="C101" s="4">
-        <v>0.3378540772532189</v>
+        <v>0.3320171673819742</v>
       </c>
       <c r="D101" s="4">
-        <v>0.9994212962962962</v>
+        <v>0.9990162037037036</v>
       </c>
       <c r="E101" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F101" s="5">
-        <v>0.8398576512455517</v>
+        <v>0.302491103202847</v>
       </c>
       <c r="G101" s="5">
-        <v>0.3430042918454935</v>
+        <v>0.3093562231759657</v>
       </c>
       <c r="H101" s="5">
-        <v>0.9826967592592591</v>
+        <v>0.9532407407407408</v>
       </c>
       <c r="I101" s="5">
-        <v>0.4839857651245552</v>
+        <v>-0.003558718861209953</v>
       </c>
       <c r="J101" s="5">
-        <v>0.005150214592274605</v>
+        <v>-0.02266094420600856</v>
       </c>
       <c r="K101" s="5">
-        <v>-0.01672453703703702</v>
+        <v>-0.04577546296296275</v>
       </c>
       <c r="M101" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N101" s="4">
-        <v>0.4113879003558719</v>
+        <v>0.3985765124555161</v>
       </c>
       <c r="O101" s="4">
-        <v>0.4659227467811158</v>
+        <v>0.4969957081545064</v>
       </c>
       <c r="P101" s="4">
-        <v>0.9992476851851851</v>
+        <v>0.999363425925926</v>
       </c>
       <c r="Q101" s="5" t="s">
         <v>8</v>
       </c>
       <c r="R101" s="5">
-        <v>0.9195729537366549</v>
+        <v>0.4448398576512456</v>
       </c>
       <c r="S101" s="5">
-        <v>0.5107296137339056</v>
+        <v>0.4945922746781116</v>
       </c>
       <c r="T101" s="5">
-        <v>0.8048032407407408</v>
+        <v>0.9993055555555556</v>
       </c>
       <c r="U101" s="5">
-        <v>0.508185053380783</v>
+        <v>0.0462633451957295</v>
       </c>
       <c r="V101" s="5">
-        <v>0.04480686695278974</v>
+        <v>-0.002403433476394767</v>
       </c>
       <c r="W101" s="5">
-        <v>-0.1944444444444443</v>
+        <v>-5.787037037041642E-05</v>
       </c>
     </row>
     <row r="102" spans="1:23">
@@ -3576,22 +3576,22 @@
         <v>9</v>
       </c>
       <c r="F102" s="5">
-        <v>0.4185053380782918</v>
+        <v>0.3494661921708185</v>
       </c>
       <c r="G102" s="5">
-        <v>0.9299570815450643</v>
+        <v>0.3325321888412017</v>
       </c>
       <c r="H102" s="5">
-        <v>0.8502314814814815</v>
+        <v>0.9988425925925926</v>
       </c>
       <c r="I102" s="5">
-        <v>0.06263345195729536</v>
+        <v>0.04341637010676158</v>
       </c>
       <c r="J102" s="5">
-        <v>0.5921030042918454</v>
+        <v>0.0005150214592274938</v>
       </c>
       <c r="K102" s="5">
-        <v>-0.1491898148148146</v>
+        <v>-0.0001736111111110272</v>
       </c>
       <c r="M102" s="4"/>
       <c r="N102" s="4"/>
@@ -3601,22 +3601,22 @@
         <v>9</v>
       </c>
       <c r="R102" s="5">
-        <v>0.2875444839857651</v>
+        <v>0.398576512455516</v>
       </c>
       <c r="S102" s="5">
-        <v>0.935793991416309</v>
+        <v>0.5014592274678111</v>
       </c>
       <c r="T102" s="5">
-        <v>0.9200231481481481</v>
+        <v>0.9988425925925928</v>
       </c>
       <c r="U102" s="5">
-        <v>-0.1238434163701068</v>
+        <v>-1.110223024625157E-16</v>
       </c>
       <c r="V102" s="5">
-        <v>0.4698712446351932</v>
+        <v>0.004463519313304742</v>
       </c>
       <c r="W102" s="5">
-        <v>-0.07922453703703702</v>
+        <v>-0.0005208333333331927</v>
       </c>
     </row>
   </sheetData>
@@ -4366,37 +4366,37 @@
         <v>8</v>
       </c>
       <c r="B6" s="4">
-        <v>106.223797750473</v>
+        <v>65.46634759902955</v>
       </c>
       <c r="C6" s="4">
-        <v>0.08531718754768372</v>
+        <v>0.05393575344085694</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E6" s="5">
-        <v>111.3706830978394</v>
+        <v>10.07893080711365</v>
       </c>
       <c r="F6" s="5">
-        <v>0.3362909124467839</v>
+        <v>0.09255615711212159</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J6" s="4">
-        <v>111.7600316047669</v>
+        <v>78.01592574119567</v>
       </c>
       <c r="K6" s="4">
-        <v>0.08994673381539964</v>
+        <v>0.06399819984436035</v>
       </c>
       <c r="L6" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M6" s="5">
-        <v>324.2510901927948</v>
+        <v>28.72236003875732</v>
       </c>
       <c r="N6" s="5">
-        <v>0.3809908160037957</v>
+        <v>0.2734680662155151</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -4407,10 +4407,10 @@
         <v>10</v>
       </c>
       <c r="E7" s="5">
-        <v>204.2996528625488</v>
+        <v>4.903269243240357</v>
       </c>
       <c r="F7" s="5">
-        <v>0.2516066266284166</v>
+        <v>0.04021444845199585</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -4419,10 +4419,10 @@
         <v>10</v>
       </c>
       <c r="M7" s="5">
-        <v>123.9222368717194</v>
+        <v>7.007123422622681</v>
       </c>
       <c r="N7" s="5">
-        <v>0.2633827979266051</v>
+        <v>0.05570521020889282</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -4430,37 +4430,37 @@
         <v>9</v>
       </c>
       <c r="B8" s="4">
-        <v>358.1482746601105</v>
+        <v>197.5463549137116</v>
       </c>
       <c r="C8" s="4">
-        <v>0.3602704426607092</v>
+        <v>0.2057124670725349</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="5">
-        <v>98.51857376098633</v>
+        <v>4.803798246383667</v>
       </c>
       <c r="F8" s="5">
-        <v>0.08008150305747984</v>
+        <v>0.004764793491363526</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J8" s="4">
-        <v>57.71408076286316</v>
+        <v>38.36131658554077</v>
       </c>
       <c r="K8" s="4">
-        <v>0.09848957090933444</v>
+        <v>0.06582506193627077</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M8" s="5">
-        <v>63.87226257324219</v>
+        <v>4.448572874069214</v>
       </c>
       <c r="N8" s="5">
-        <v>0.04350452332496643</v>
+        <v>0.006802116147933468</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -4471,10 +4471,10 @@
         <v>10</v>
       </c>
       <c r="E9" s="5">
-        <v>139.2045318603516</v>
+        <v>7.890654134750366</v>
       </c>
       <c r="F9" s="5">
-        <v>0.4833147639807902</v>
+        <v>0.06981702661514283</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" s="4"/>
@@ -4483,10 +4483,10 @@
         <v>10</v>
       </c>
       <c r="M9" s="5">
-        <v>409.1327763080597</v>
+        <v>6.718277025222778</v>
       </c>
       <c r="N9" s="5">
-        <v>1.037597999903216</v>
+        <v>0.05390745735168458</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -4494,37 +4494,37 @@
         <v>10</v>
       </c>
       <c r="B10" s="4">
-        <v>307.6326349258423</v>
+        <v>155.981974029541</v>
       </c>
       <c r="C10" s="4">
-        <v>1.021092890450792</v>
+        <v>0.582466755995487</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="5">
-        <v>89.48915648460388</v>
+        <v>1.529009532928467</v>
       </c>
       <c r="F10" s="5">
-        <v>0.07264830961227417</v>
+        <v>0.007139796257019044</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J10" s="4">
-        <v>164.361366558075</v>
+        <v>124.9881973266602</v>
       </c>
       <c r="K10" s="4">
-        <v>0.2886743840133753</v>
+        <v>0.201352038398224</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M10" s="5">
-        <v>42.84506125450135</v>
+        <v>1.942640113830566</v>
       </c>
       <c r="N10" s="5">
-        <v>0.0382739151969048</v>
+        <v>0.006420305728912354</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -4535,10 +4535,10 @@
         <v>9</v>
       </c>
       <c r="E11" s="5">
-        <v>138.8495800971985</v>
+        <v>19.25746250152588</v>
       </c>
       <c r="F11" s="5">
-        <v>0.1506451794890973</v>
+        <v>0.1842250618934632</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" s="4"/>
@@ -4547,10 +4547,10 @@
         <v>9</v>
       </c>
       <c r="M11" s="5">
-        <v>163.9307970523834</v>
+        <v>26.59402189254761</v>
       </c>
       <c r="N11" s="5">
-        <v>0.1618762058344027</v>
+        <v>0.2526897478103638</v>
       </c>
     </row>
     <row r="18" spans="1:14">
@@ -4644,37 +4644,37 @@
         <v>8</v>
       </c>
       <c r="B21" s="4">
-        <v>115.1382991790772</v>
+        <v>76.56184659004211</v>
       </c>
       <c r="C21" s="4">
-        <v>0.09225407443046571</v>
+        <v>0.06284926896095275</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E21" s="5">
-        <v>286.798372888565</v>
+        <v>3.497618627548218</v>
       </c>
       <c r="F21" s="5">
-        <v>0.3659940032920321</v>
+        <v>0.02082125663757324</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J21" s="4">
-        <v>120.9741519927979</v>
+        <v>75.00341415405273</v>
       </c>
       <c r="K21" s="4">
-        <v>0.1029577269559063</v>
+        <v>0.06285679540617579</v>
       </c>
       <c r="L21" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M21" s="5">
-        <v>58.13424568176269</v>
+        <v>3.507832384109497</v>
       </c>
       <c r="N21" s="5">
-        <v>0.2399064791041528</v>
+        <v>0.02037670564651489</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -4685,10 +4685,10 @@
         <v>10</v>
       </c>
       <c r="E22" s="5">
-        <v>200.2699111461639</v>
+        <v>6.486885404586792</v>
       </c>
       <c r="F22" s="5">
-        <v>1.101843554290034</v>
+        <v>0.05123506069183349</v>
       </c>
       <c r="I22" s="4"/>
       <c r="J22" s="4"/>
@@ -4697,10 +4697,10 @@
         <v>10</v>
       </c>
       <c r="M22" s="5">
-        <v>180.1982127666473</v>
+        <v>6.965536403656006</v>
       </c>
       <c r="N22" s="5">
-        <v>0.1806296310143607</v>
+        <v>0.0551024832725525</v>
       </c>
     </row>
     <row r="23" spans="1:14">
@@ -4708,37 +4708,37 @@
         <v>9</v>
       </c>
       <c r="B23" s="4">
-        <v>149.0787490367889</v>
+        <v>113.7783089160919</v>
       </c>
       <c r="C23" s="4">
-        <v>0.3877672752793967</v>
+        <v>0.2301089025614757</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="5">
-        <v>109.4321567058563</v>
+        <v>2.276444292068482</v>
       </c>
       <c r="F23" s="5">
-        <v>0.09006798147409349</v>
+        <v>0.006037412832180659</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J23" s="4">
-        <v>45.11588163375855</v>
+        <v>20.17258858680725</v>
       </c>
       <c r="K23" s="4">
-        <v>0.1199198021871859</v>
+        <v>0.06829983490886264</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M23" s="5">
-        <v>74.39385604858398</v>
+        <v>2.217529439926147</v>
       </c>
       <c r="N23" s="5">
-        <v>0.05470164475359608</v>
+        <v>0.007255810737609864</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -4749,10 +4749,10 @@
         <v>10</v>
       </c>
       <c r="E24" s="5">
-        <v>191.5058953762054</v>
+        <v>34.57574119567871</v>
       </c>
       <c r="F24" s="5">
-        <v>1.064896763576061</v>
+        <v>0.333575098991394</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" s="4"/>
@@ -4761,10 +4761,10 @@
         <v>10</v>
       </c>
       <c r="M24" s="5">
-        <v>172.5256417274475</v>
+        <v>6.564522123336792</v>
       </c>
       <c r="N24" s="5">
-        <v>0.3333247978708439</v>
+        <v>0.05230565595626831</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -4772,37 +4772,37 @@
         <v>10</v>
       </c>
       <c r="B25" s="4">
-        <v>183.2678444862366</v>
+        <v>104.6178802967072</v>
       </c>
       <c r="C25" s="4">
-        <v>0.3055105255388078</v>
+        <v>0.1746090329719102</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E25" s="5">
-        <v>99.46511759757996</v>
+        <v>1.939098405838013</v>
       </c>
       <c r="F25" s="5">
-        <v>0.08547790536220891</v>
+        <v>0.006331727027893067</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J25" s="4">
-        <v>282.9510268688202</v>
+        <v>170.4672595977783</v>
       </c>
       <c r="K25" s="4">
-        <v>0.3526043985127866</v>
+        <v>0.200172061400031</v>
       </c>
       <c r="L25" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M25" s="5">
-        <v>58.62762680053711</v>
+        <v>4.44277081489563</v>
       </c>
       <c r="N25" s="5">
-        <v>0.1009884846627384</v>
+        <v>0.03169587659835815</v>
       </c>
     </row>
     <row r="26" spans="1:14">
@@ -4813,10 +4813,10 @@
         <v>9</v>
       </c>
       <c r="E26" s="5">
-        <v>123.8191955566406</v>
+        <v>22.95618414878845</v>
       </c>
       <c r="F26" s="5">
-        <v>0.3359572430377833</v>
+        <v>0.2175214724540711</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" s="4"/>
@@ -4825,10 +4825,10 @@
         <v>9</v>
       </c>
       <c r="M26" s="5">
-        <v>255.3079745769501</v>
+        <v>3.264210844039917</v>
       </c>
       <c r="N26" s="5">
-        <v>0.4067184279255307</v>
+        <v>0.01925837421417236</v>
       </c>
     </row>
     <row r="33" spans="1:14">
@@ -4922,37 +4922,37 @@
         <v>8</v>
       </c>
       <c r="B36" s="4">
-        <v>118.1840867519379</v>
+        <v>75.99118499755859</v>
       </c>
       <c r="C36" s="4">
-        <v>0.09461622953414917</v>
+        <v>0.06213307642936707</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E36" s="5">
-        <v>252.7342121601105</v>
+        <v>2.936468696594238</v>
       </c>
       <c r="F36" s="5">
-        <v>0.380370298679413</v>
+        <v>0.01750487375259399</v>
       </c>
       <c r="I36" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J36" s="4">
-        <v>93.06554803848266</v>
+        <v>51.91652693748474</v>
       </c>
       <c r="K36" s="4">
-        <v>0.08069747352745857</v>
+        <v>0.05478188028759255</v>
       </c>
       <c r="L36" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M36" s="5">
-        <v>43.95318398475647</v>
+        <v>18.17486581802368</v>
       </c>
       <c r="N36" s="5">
-        <v>0.1670453131984634</v>
+        <v>0.173071448802948</v>
       </c>
     </row>
     <row r="37" spans="1:14">
@@ -4963,10 +4963,10 @@
         <v>10</v>
       </c>
       <c r="E37" s="5">
-        <v>183.4072152137756</v>
+        <v>5.802566146850586</v>
       </c>
       <c r="F37" s="5">
-        <v>0.5472923959191476</v>
+        <v>0.04607759571075439</v>
       </c>
       <c r="I37" s="4"/>
       <c r="J37" s="4"/>
@@ -4975,10 +4975,10 @@
         <v>10</v>
       </c>
       <c r="M37" s="5">
-        <v>481.0381036281586</v>
+        <v>4.603079462051392</v>
       </c>
       <c r="N37" s="5">
-        <v>0.4854540395596483</v>
+        <v>0.0375020112991333</v>
       </c>
     </row>
     <row r="38" spans="1:14">
@@ -4986,37 +4986,37 @@
         <v>9</v>
       </c>
       <c r="B38" s="4">
-        <v>229.4624054431915</v>
+        <v>157.2831580162048</v>
       </c>
       <c r="C38" s="4">
-        <v>0.391254064264039</v>
+        <v>0.2194775407715474</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E38" s="5">
-        <v>111.3983274936676</v>
+        <v>2.301779270172119</v>
       </c>
       <c r="F38" s="5">
-        <v>0.08993294591903686</v>
+        <v>0.01029643249511719</v>
       </c>
       <c r="I38" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J38" s="4">
-        <v>32.96514449119568</v>
+        <v>14.07423467636108</v>
       </c>
       <c r="K38" s="4">
-        <v>0.02707017606647713</v>
+        <v>0.01691407094574145</v>
       </c>
       <c r="L38" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M38" s="5">
-        <v>23.65061464309692</v>
+        <v>5.313333845138549</v>
       </c>
       <c r="N38" s="5">
-        <v>0.01796240511668783</v>
+        <v>0.005433080843554899</v>
       </c>
     </row>
     <row r="39" spans="1:14">
@@ -5027,10 +5027,10 @@
         <v>10</v>
       </c>
       <c r="E39" s="5">
-        <v>175.9163191795349</v>
+        <v>5.948477506637573</v>
       </c>
       <c r="F39" s="5">
-        <v>1.079984780904198</v>
+        <v>0.04699403381347656</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" s="4"/>
@@ -5039,10 +5039,10 @@
         <v>10</v>
       </c>
       <c r="M39" s="5">
-        <v>154.2967624664307</v>
+        <v>4.569569301605225</v>
       </c>
       <c r="N39" s="5">
-        <v>0.4346355288388798</v>
+        <v>0.03707122039794921</v>
       </c>
     </row>
     <row r="40" spans="1:14">
@@ -5050,37 +5050,37 @@
         <v>10</v>
       </c>
       <c r="B40" s="4">
-        <v>224.2051598548889</v>
+        <v>108.4320956230164</v>
       </c>
       <c r="C40" s="4">
-        <v>0.6108048924557241</v>
+        <v>0.3413240107720406</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E40" s="5">
-        <v>75.124387216568</v>
+        <v>1.963647413253784</v>
       </c>
       <c r="F40" s="5">
-        <v>0.08727695665269571</v>
+        <v>0.005662329678978424</v>
       </c>
       <c r="I40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J40" s="4">
-        <v>659.2631187915802</v>
+        <v>355.7323093414307</v>
       </c>
       <c r="K40" s="4">
-        <v>1.012753832314657</v>
+        <v>0.5665015714268067</v>
       </c>
       <c r="L40" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M40" s="5">
-        <v>37.94477953910827</v>
+        <v>5.135971879959106</v>
       </c>
       <c r="N40" s="5">
-        <v>0.07094480623584429</v>
+        <v>0.04277742147445679</v>
       </c>
     </row>
     <row r="41" spans="1:14">
@@ -5091,10 +5091,10 @@
         <v>9</v>
       </c>
       <c r="E41" s="5">
-        <v>101.8805916309357</v>
+        <v>2.805486583709717</v>
       </c>
       <c r="F41" s="5">
-        <v>0.1754038376405481</v>
+        <v>0.01650038003921509</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" s="4"/>
@@ -5103,10 +5103,10 @@
         <v>9</v>
       </c>
       <c r="M41" s="5">
-        <v>27.92054023742676</v>
+        <v>5.560752630233765</v>
       </c>
       <c r="N41" s="5">
-        <v>0.140649820606792</v>
+        <v>0.04705390501022339</v>
       </c>
     </row>
     <row r="48" spans="1:14">
@@ -5200,37 +5200,37 @@
         <v>8</v>
       </c>
       <c r="B51" s="4">
-        <v>100.0630198001862</v>
+        <v>60.80864734649658</v>
       </c>
       <c r="C51" s="4">
-        <v>0.1052956309825493</v>
+        <v>0.06520130118531232</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E51" s="5">
-        <v>182.0247549533844</v>
+        <v>9.169482803344726</v>
       </c>
       <c r="F51" s="5">
-        <v>0.4737248064775278</v>
+        <v>0.07571729755401611</v>
       </c>
       <c r="I51" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J51" s="4">
-        <v>127.2557045459747</v>
+        <v>71.75876107215882</v>
       </c>
       <c r="K51" s="4">
-        <v>0.1086654386543929</v>
+        <v>0.06160325256944539</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M51" s="5">
-        <v>151.4744189739227</v>
+        <v>25.50445170402527</v>
       </c>
       <c r="N51" s="5">
-        <v>0.2355664508304862</v>
+        <v>0.240275990847245</v>
       </c>
     </row>
     <row r="52" spans="1:14">
@@ -5241,10 +5241,10 @@
         <v>10</v>
       </c>
       <c r="E52" s="5">
-        <v>143.5127764225006</v>
+        <v>7.494287204742432</v>
       </c>
       <c r="F52" s="5">
-        <v>1.405753026008606</v>
+        <v>0.0588059482574463</v>
       </c>
       <c r="I52" s="4"/>
       <c r="J52" s="4"/>
@@ -5253,10 +5253,10 @@
         <v>10</v>
       </c>
       <c r="M52" s="5">
-        <v>139.5842367649078</v>
+        <v>6.930582427978516</v>
       </c>
       <c r="N52" s="5">
-        <v>0.7044119646254076</v>
+        <v>0.05409246301651001</v>
       </c>
     </row>
     <row r="53" spans="1:14">
@@ -5264,37 +5264,37 @@
         <v>9</v>
       </c>
       <c r="B53" s="4">
-        <v>119.5429006099701</v>
+        <v>64.93307161331177</v>
       </c>
       <c r="C53" s="4">
-        <v>0.4659292459473205</v>
+        <v>0.2499458561021813</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E53" s="5">
-        <v>121.6206075668335</v>
+        <v>3.146953153610229</v>
       </c>
       <c r="F53" s="5">
-        <v>0.1124930221367804</v>
+        <v>0.01754777479171753</v>
       </c>
       <c r="I53" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J53" s="4">
-        <v>105.86143450737</v>
+        <v>55.35616097450256</v>
       </c>
       <c r="K53" s="4">
-        <v>0.2298168027495849</v>
+        <v>0.133561590140846</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M53" s="5">
-        <v>113.9527386188507</v>
+        <v>2.0312912940979</v>
       </c>
       <c r="N53" s="5">
-        <v>0.1126977162087966</v>
+        <v>0.006363752365112304</v>
       </c>
     </row>
     <row r="54" spans="1:14">
@@ -5305,10 +5305,10 @@
         <v>10</v>
       </c>
       <c r="E54" s="5">
-        <v>150.8710789680481</v>
+        <v>21.70537724494934</v>
       </c>
       <c r="F54" s="5">
-        <v>1.357300905508729</v>
+        <v>0.2021080455780029</v>
       </c>
       <c r="I54" s="4"/>
       <c r="J54" s="4"/>
@@ -5317,10 +5317,10 @@
         <v>10</v>
       </c>
       <c r="M54" s="5">
-        <v>159.9670229434967</v>
+        <v>68.02584824562072</v>
       </c>
       <c r="N54" s="5">
-        <v>1.382224915539239</v>
+        <v>0.6668027925491333</v>
       </c>
     </row>
     <row r="55" spans="1:14">
@@ -5328,37 +5328,37 @@
         <v>10</v>
       </c>
       <c r="B55" s="4">
-        <v>141.7108589172363</v>
+        <v>77.55571246147156</v>
       </c>
       <c r="C55" s="4">
-        <v>1.388055045604706</v>
+        <v>0.7604588537216187</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E55" s="5">
-        <v>109.0908139228821</v>
+        <v>8.174049425125123</v>
       </c>
       <c r="F55" s="5">
-        <v>0.1143900647236431</v>
+        <v>0.06715331554412843</v>
       </c>
       <c r="I55" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J55" s="4">
-        <v>143.9834718704224</v>
+        <v>76.64656190872192</v>
       </c>
       <c r="K55" s="4">
-        <v>1.410171739578247</v>
+        <v>0.7517248325347901</v>
       </c>
       <c r="L55" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M55" s="5">
-        <v>126.9342513084412</v>
+        <v>1.967167949676514</v>
       </c>
       <c r="N55" s="5">
-        <v>0.1137439252118783</v>
+        <v>0.006328228473663331</v>
       </c>
     </row>
     <row r="56" spans="1:14">
@@ -5369,10 +5369,10 @@
         <v>9</v>
       </c>
       <c r="E56" s="5">
-        <v>153.5690554618836</v>
+        <v>8.893216323852538</v>
       </c>
       <c r="F56" s="5">
-        <v>0.448579639516772</v>
+        <v>0.0738379783630371</v>
       </c>
       <c r="I56" s="4"/>
       <c r="J56" s="4"/>
@@ -5381,10 +5381,10 @@
         <v>9</v>
       </c>
       <c r="M56" s="5">
-        <v>138.6753211021423</v>
+        <v>3.135001707077026</v>
       </c>
       <c r="N56" s="5">
-        <v>0.4537981230948789</v>
+        <v>0.01844130897521973</v>
       </c>
     </row>
     <row r="63" spans="1:14">
@@ -5478,37 +5478,37 @@
         <v>8</v>
       </c>
       <c r="B66" s="4">
-        <v>7.190635299682617</v>
+        <v>8.083817052841187</v>
       </c>
       <c r="C66" s="4">
-        <v>0.0281525228233535</v>
+        <v>0.01546750845909119</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E66" s="5">
-        <v>135.3377210140228</v>
+        <v>3.172017478942871</v>
       </c>
       <c r="F66" s="5">
-        <v>0.249755525831872</v>
+        <v>0.01851664781570435</v>
       </c>
       <c r="I66" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J66" s="4">
-        <v>144.1305657863617</v>
+        <v>77.60522847175598</v>
       </c>
       <c r="K66" s="4">
-        <v>0.11663299489462</v>
+        <v>0.06360148798326833</v>
       </c>
       <c r="L66" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M66" s="5">
-        <v>16.68098812103272</v>
+        <v>3.321150112152099</v>
       </c>
       <c r="N66" s="5">
-        <v>0.1343578314781189</v>
+        <v>0.01910228681564331</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -5519,10 +5519,10 @@
         <v>10</v>
       </c>
       <c r="E67" s="5">
-        <v>163.4750289440155</v>
+        <v>6.032295513153076</v>
       </c>
       <c r="F67" s="5">
-        <v>1.561618477121717</v>
+        <v>0.04673698091506957</v>
       </c>
       <c r="I67" s="4"/>
       <c r="J67" s="4"/>
@@ -5531,10 +5531,10 @@
         <v>10</v>
       </c>
       <c r="M67" s="5">
-        <v>201.7852386951446</v>
+        <v>71.78062801361084</v>
       </c>
       <c r="N67" s="5">
-        <v>1.523004842114169</v>
+        <v>0.7040735068321228</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -5542,37 +5542,37 @@
         <v>9</v>
       </c>
       <c r="B68" s="4">
-        <v>96.50624356269836</v>
+        <v>44.79288473129272</v>
       </c>
       <c r="C68" s="4">
-        <v>0.4682127485852218</v>
+        <v>0.2567768927307769</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E68" s="5">
-        <v>6.598030567169189</v>
+        <v>8.272517013549805</v>
       </c>
       <c r="F68" s="5">
-        <v>0.03076681313795202</v>
+        <v>0.06806587982177734</v>
       </c>
       <c r="I68" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J68" s="4">
-        <v>54.73321137428284</v>
+        <v>27.77803773880005</v>
       </c>
       <c r="K68" s="4">
-        <v>0.5157132868766784</v>
+        <v>0.262634355545044</v>
       </c>
       <c r="L68" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M68" s="5">
-        <v>137.5000148296356</v>
+        <v>7.079879522323608</v>
       </c>
       <c r="N68" s="5">
-        <v>0.1221594133817844</v>
+        <v>0.05822457742691041</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -5583,10 +5583,10 @@
         <v>10</v>
       </c>
       <c r="E69" s="5">
-        <v>162.8909076690674</v>
+        <v>81.58644871711731</v>
       </c>
       <c r="F69" s="5">
-        <v>1.545288358211517</v>
+        <v>0.7997959785461426</v>
       </c>
       <c r="I69" s="4"/>
       <c r="J69" s="4"/>
@@ -5595,10 +5595,10 @@
         <v>10</v>
       </c>
       <c r="M69" s="5">
-        <v>153.5959408283234</v>
+        <v>34.81821293830872</v>
       </c>
       <c r="N69" s="5">
-        <v>0.3586401372575063</v>
+        <v>0.3354621825218201</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -5606,37 +5606,37 @@
         <v>10</v>
       </c>
       <c r="B70" s="4">
-        <v>156.2532437324524</v>
+        <v>76.01525521278381</v>
       </c>
       <c r="C70" s="4">
-        <v>1.530882461547852</v>
+        <v>0.7407829085507439</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E70" s="5">
-        <v>4.996485614776612</v>
+        <v>8.089029693603516</v>
       </c>
       <c r="F70" s="5">
-        <v>0.01248064315013396</v>
+        <v>0.06671871232986451</v>
       </c>
       <c r="I70" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J70" s="4">
-        <v>155.641857624054</v>
+        <v>77.80746378898621</v>
       </c>
       <c r="K70" s="4">
-        <v>1.524672620773315</v>
+        <v>0.7610334781656171</v>
       </c>
       <c r="L70" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M70" s="5">
-        <v>124.158872461319</v>
+        <v>1.715272426605225</v>
       </c>
       <c r="N70" s="5">
-        <v>0.1183393508976748</v>
+        <v>0.005709434509277344</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -5647,10 +5647,10 @@
         <v>9</v>
       </c>
       <c r="E71" s="5">
-        <v>171.8918225765228</v>
+        <v>14.8980366230011</v>
       </c>
       <c r="F71" s="5">
-        <v>0.5232989887350671</v>
+        <v>0.1347329602241516</v>
       </c>
       <c r="I71" s="4"/>
       <c r="J71" s="4"/>
@@ -5659,10 +5659,10 @@
         <v>9</v>
       </c>
       <c r="M71" s="5">
-        <v>32.63117022514344</v>
+        <v>4.585118675231934</v>
       </c>
       <c r="N71" s="5">
-        <v>0.03545062956809997</v>
+        <v>0.03255372238159179</v>
       </c>
     </row>
     <row r="78" spans="1:14">
@@ -5756,37 +5756,37 @@
         <v>8</v>
       </c>
       <c r="B81" s="4">
-        <v>8.975301837921142</v>
+        <v>5.105287361145019</v>
       </c>
       <c r="C81" s="4">
-        <v>0.05478035939845226</v>
+        <v>0.0310475866776874</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>9</v>
       </c>
       <c r="E81" s="5">
-        <v>100.5157667160034</v>
+        <v>46.523650598526</v>
       </c>
       <c r="F81" s="5">
-        <v>0.9767852063179017</v>
+        <v>0.4565883998870849</v>
       </c>
       <c r="I81" s="4" t="s">
         <v>8</v>
       </c>
       <c r="J81" s="4">
-        <v>95.94409170150757</v>
+        <v>78.84259743690491</v>
       </c>
       <c r="K81" s="4">
-        <v>0.1721524163336317</v>
+        <v>0.1123490397672996</v>
       </c>
       <c r="L81" s="5" t="s">
         <v>9</v>
       </c>
       <c r="M81" s="5">
-        <v>108.8621156692505</v>
+        <v>3.566619825363159</v>
       </c>
       <c r="N81" s="5">
-        <v>0.185000655666485</v>
+        <v>0.02843578004837036</v>
       </c>
     </row>
     <row r="82" spans="1:14">
@@ -5797,10 +5797,10 @@
         <v>10</v>
       </c>
       <c r="E82" s="5">
-        <v>305.3393357753754</v>
+        <v>138.6971946716309</v>
       </c>
       <c r="F82" s="5">
-        <v>2.929224489045667</v>
+        <v>1.377534533023834</v>
       </c>
       <c r="I82" s="4"/>
       <c r="J82" s="4"/>
@@ -5809,10 +5809,10 @@
         <v>10</v>
       </c>
       <c r="M82" s="5">
-        <v>527.5165868759156</v>
+        <v>8.325389385223389</v>
       </c>
       <c r="N82" s="5">
-        <v>0.5362185416052732</v>
+        <v>0.07683311653137206</v>
       </c>
     </row>
     <row r="83" spans="1:14">
@@ -5820,37 +5820,37 @@
         <v>9</v>
       </c>
       <c r="B83" s="4">
-        <v>98.27692966461181</v>
+        <v>49.58945617675781</v>
       </c>
       <c r="C83" s="4">
-        <v>0.9545185565948486</v>
+        <v>0.4863302283287048</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E83" s="5">
-        <v>17.33097615242004</v>
+        <v>11.57184715270996</v>
       </c>
       <c r="F83" s="5">
-        <v>0.1277314852293879</v>
+        <v>0.1083170161247254</v>
       </c>
       <c r="I83" s="4" t="s">
         <v>9</v>
       </c>
       <c r="J83" s="4">
-        <v>83.9740282535553</v>
+        <v>50.20753889083862</v>
       </c>
       <c r="K83" s="4">
-        <v>0.8119552412572897</v>
+        <v>0.4502992669190909</v>
       </c>
       <c r="L83" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M83" s="5">
-        <v>19.25290021896362</v>
+        <v>10.80864229202271</v>
       </c>
       <c r="N83" s="5">
-        <v>0.1680337904271519</v>
+        <v>0.1017983021736145</v>
       </c>
     </row>
     <row r="84" spans="1:14">
@@ -5861,10 +5861,10 @@
         <v>10</v>
       </c>
       <c r="E84" s="5">
-        <v>164.7753010749817</v>
+        <v>33.39773740768432</v>
       </c>
       <c r="F84" s="5">
-        <v>1.457247624573544</v>
+        <v>0.3258714776039124</v>
       </c>
       <c r="I84" s="4"/>
       <c r="J84" s="4"/>
@@ -5873,10 +5873,10 @@
         <v>10</v>
       </c>
       <c r="M84" s="5">
-        <v>209.8068177700043</v>
+        <v>61.92241659164429</v>
       </c>
       <c r="N84" s="5">
-        <v>1.932443463409082</v>
+        <v>0.6037496366134057</v>
       </c>
     </row>
     <row r="85" spans="1:14">
@@ -5884,37 +5884,37 @@
         <v>10</v>
       </c>
       <c r="B85" s="4">
-        <v>318.6029125213623</v>
+        <v>145.7722337722778</v>
       </c>
       <c r="C85" s="4">
-        <v>2.874112078705638</v>
+        <v>1.393815158057631</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E85" s="5">
-        <v>33.76639785766601</v>
+        <v>9.380964422225953</v>
       </c>
       <c r="F85" s="5">
-        <v>0.2356843034416816</v>
+        <v>0.05464633186832012</v>
       </c>
       <c r="I85" s="4" t="s">
         <v>10</v>
       </c>
       <c r="J85" s="4">
-        <v>233.7937679290771</v>
+        <v>131.9877051353455</v>
       </c>
       <c r="K85" s="4">
-        <v>2.230621384288225</v>
+        <v>1.277426834063097</v>
       </c>
       <c r="L85" s="5" t="s">
         <v>8</v>
       </c>
       <c r="M85" s="5">
-        <v>11.30035533905029</v>
+        <v>1.98493390083313</v>
       </c>
       <c r="N85" s="5">
-        <v>0.07819871700884214</v>
+        <v>0.01332335898172941</v>
       </c>
     </row>
     <row r="86" spans="1:14">
@@ -5925,10 +5925,10 @@
         <v>9</v>
       </c>
       <c r="E86" s="5">
-        <v>48.88521642684937</v>
+        <v>45.67915616035462</v>
       </c>
       <c r="F86" s="5">
-        <v>0.4616946840286255</v>
+        <v>0.4225346933514619</v>
       </c>
       <c r="I86" s="4"/>
       <c r="J86" s="4"/>
@@ -5937,10 +5937,10 @@
         <v>9</v>
       </c>
       <c r="M86" s="5">
-        <v>16.60587015151977</v>
+        <v>39.74485020637512</v>
       </c>
       <c r="N86" s="5">
-        <v>0.1512543630599976</v>
+        <v>0.3914464702606201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>